<commit_message>
Plate reader kinetics: green/yellow/red tint for trace quality, restore notes; stronger depletion in practice plate
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0162t2pqYZEZsR9bb7f2rWiV
</commit_message>
<xml_diff>
--- a/examples/practice_plate_simulated.xlsx
+++ b/examples/practice_plate_simulated.xlsx
@@ -1055,109 +1055,109 @@
         <v>0.2015</v>
       </c>
       <c r="D37" t="n">
-        <v>0.2404</v>
+        <v>0.2405</v>
       </c>
       <c r="E37" t="n">
-        <v>0.2752</v>
+        <v>0.2753</v>
       </c>
       <c r="F37" t="n">
-        <v>0.3147</v>
+        <v>0.3149</v>
       </c>
       <c r="G37" t="n">
-        <v>0.3503</v>
+        <v>0.3506</v>
       </c>
       <c r="H37" t="n">
-        <v>0.3875</v>
+        <v>0.3878</v>
       </c>
       <c r="I37" t="n">
-        <v>0.4217</v>
+        <v>0.4221</v>
       </c>
       <c r="J37" t="n">
-        <v>0.4626</v>
+        <v>0.463</v>
       </c>
       <c r="K37" t="n">
-        <v>0.4977</v>
+        <v>0.4982</v>
       </c>
       <c r="L37" t="n">
-        <v>0.533</v>
+        <v>0.5335</v>
       </c>
       <c r="M37" t="n">
-        <v>0.5718</v>
+        <v>0.5724</v>
       </c>
       <c r="N37" t="n">
-        <v>0.6055</v>
+        <v>0.6062</v>
       </c>
       <c r="O37" t="n">
-        <v>0.6423</v>
+        <v>0.643</v>
       </c>
       <c r="P37" t="n">
-        <v>0.6804</v>
+        <v>0.6812</v>
       </c>
       <c r="Q37" t="n">
-        <v>0.7171999999999999</v>
+        <v>0.718</v>
       </c>
       <c r="R37" t="n">
-        <v>0.7514</v>
+        <v>0.7524</v>
       </c>
       <c r="S37" t="n">
-        <v>0.7881</v>
+        <v>0.789</v>
       </c>
       <c r="T37" t="n">
-        <v>0.8221000000000001</v>
+        <v>0.8232</v>
       </c>
       <c r="U37" t="n">
-        <v>0.8597</v>
+        <v>0.8608</v>
       </c>
       <c r="V37" t="n">
-        <v>0.8904</v>
+        <v>0.8915</v>
       </c>
       <c r="W37" t="n">
-        <v>0.9349</v>
+        <v>0.9361</v>
       </c>
       <c r="X37" t="n">
-        <v>0.9637</v>
+        <v>0.9649</v>
       </c>
       <c r="Y37" t="n">
-        <v>0.9981</v>
+        <v>0.9994</v>
       </c>
       <c r="Z37" t="n">
-        <v>1.032</v>
+        <v>1.0333</v>
       </c>
       <c r="AA37" t="n">
-        <v>1.069</v>
+        <v>1.0704</v>
       </c>
       <c r="AB37" t="n">
-        <v>1.101</v>
+        <v>1.1025</v>
       </c>
       <c r="AC37" t="n">
-        <v>1.1392</v>
+        <v>1.1407</v>
       </c>
       <c r="AD37" t="n">
-        <v>1.1729</v>
+        <v>1.1744</v>
       </c>
       <c r="AE37" t="n">
-        <v>1.2037</v>
+        <v>1.2053</v>
       </c>
       <c r="AF37" t="n">
-        <v>1.2383</v>
+        <v>1.2399</v>
       </c>
       <c r="AG37" t="n">
-        <v>1.273</v>
+        <v>1.2747</v>
       </c>
       <c r="AH37" t="n">
-        <v>1.3099</v>
+        <v>1.3116</v>
       </c>
       <c r="AI37" t="n">
-        <v>1.3414</v>
+        <v>1.3431</v>
       </c>
       <c r="AJ37" t="n">
-        <v>1.372</v>
+        <v>1.3738</v>
       </c>
       <c r="AK37" t="n">
-        <v>1.4091</v>
+        <v>1.4109</v>
       </c>
       <c r="AL37" t="n">
-        <v>1.4523</v>
+        <v>1.4543</v>
       </c>
     </row>
     <row r="38">
@@ -1173,109 +1173,109 @@
         <v>0.1906</v>
       </c>
       <c r="D38" t="n">
-        <v>0.2067</v>
+        <v>0.2068</v>
       </c>
       <c r="E38" t="n">
-        <v>0.2333</v>
+        <v>0.2334</v>
       </c>
       <c r="F38" t="n">
-        <v>0.2613</v>
+        <v>0.2616</v>
       </c>
       <c r="G38" t="n">
-        <v>0.2959</v>
+        <v>0.2963</v>
       </c>
       <c r="H38" t="n">
-        <v>0.333</v>
+        <v>0.3336</v>
       </c>
       <c r="I38" t="n">
-        <v>0.37</v>
+        <v>0.3707</v>
       </c>
       <c r="J38" t="n">
-        <v>0.4097</v>
+        <v>0.4105</v>
       </c>
       <c r="K38" t="n">
-        <v>0.4497</v>
+        <v>0.4506</v>
       </c>
       <c r="L38" t="n">
-        <v>0.4907</v>
+        <v>0.4918</v>
       </c>
       <c r="M38" t="n">
-        <v>0.5327</v>
+        <v>0.5339</v>
       </c>
       <c r="N38" t="n">
-        <v>0.5743</v>
+        <v>0.5757</v>
       </c>
       <c r="O38" t="n">
-        <v>0.6155</v>
+        <v>0.617</v>
       </c>
       <c r="P38" t="n">
-        <v>0.6562</v>
+        <v>0.6579</v>
       </c>
       <c r="Q38" t="n">
-        <v>0.6965</v>
+        <v>0.6982</v>
       </c>
       <c r="R38" t="n">
-        <v>0.7377</v>
+        <v>0.7396</v>
       </c>
       <c r="S38" t="n">
-        <v>0.781</v>
+        <v>0.7831</v>
       </c>
       <c r="T38" t="n">
-        <v>0.8216</v>
+        <v>0.8238</v>
       </c>
       <c r="U38" t="n">
-        <v>0.8611</v>
+        <v>0.8633999999999999</v>
       </c>
       <c r="V38" t="n">
-        <v>0.9015</v>
+        <v>0.9039</v>
       </c>
       <c r="W38" t="n">
-        <v>0.9472</v>
+        <v>0.9498</v>
       </c>
       <c r="X38" t="n">
-        <v>0.9848</v>
+        <v>0.9875</v>
       </c>
       <c r="Y38" t="n">
-        <v>1.0242</v>
+        <v>1.027</v>
       </c>
       <c r="Z38" t="n">
-        <v>1.07</v>
+        <v>1.0731</v>
       </c>
       <c r="AA38" t="n">
-        <v>1.1108</v>
+        <v>1.114</v>
       </c>
       <c r="AB38" t="n">
-        <v>1.1483</v>
+        <v>1.1515</v>
       </c>
       <c r="AC38" t="n">
-        <v>1.1868</v>
+        <v>1.1903</v>
       </c>
       <c r="AD38" t="n">
-        <v>1.2294</v>
+        <v>1.233</v>
       </c>
       <c r="AE38" t="n">
-        <v>1.2745</v>
+        <v>1.2782</v>
       </c>
       <c r="AF38" t="n">
-        <v>1.3088</v>
+        <v>1.3126</v>
       </c>
       <c r="AG38" t="n">
-        <v>1.3477</v>
+        <v>1.3516</v>
       </c>
       <c r="AH38" t="n">
-        <v>1.3876</v>
+        <v>1.3916</v>
       </c>
       <c r="AI38" t="n">
-        <v>1.4277</v>
+        <v>1.4319</v>
       </c>
       <c r="AJ38" t="n">
-        <v>1.4717</v>
+        <v>1.4761</v>
       </c>
       <c r="AK38" t="n">
-        <v>1.4999</v>
+        <v>1.5043</v>
       </c>
       <c r="AL38" t="n">
-        <v>1.5444</v>
+        <v>1.549</v>
       </c>
     </row>
     <row r="39">
@@ -1288,112 +1288,112 @@
         <v>0.1856</v>
       </c>
       <c r="C39" t="n">
-        <v>0.225</v>
+        <v>0.2253</v>
       </c>
       <c r="D39" t="n">
-        <v>0.2689</v>
+        <v>0.2696</v>
       </c>
       <c r="E39" t="n">
-        <v>0.3105</v>
+        <v>0.3115</v>
       </c>
       <c r="F39" t="n">
-        <v>0.3544</v>
+        <v>0.3557</v>
       </c>
       <c r="G39" t="n">
-        <v>0.3996</v>
+        <v>0.4012</v>
       </c>
       <c r="H39" t="n">
-        <v>0.44</v>
+        <v>0.4418</v>
       </c>
       <c r="I39" t="n">
-        <v>0.483</v>
+        <v>0.4852</v>
       </c>
       <c r="J39" t="n">
-        <v>0.5268</v>
+        <v>0.5293</v>
       </c>
       <c r="K39" t="n">
-        <v>0.57</v>
+        <v>0.5728</v>
       </c>
       <c r="L39" t="n">
-        <v>0.6139</v>
+        <v>0.6171</v>
       </c>
       <c r="M39" t="n">
-        <v>0.6556999999999999</v>
+        <v>0.6592</v>
       </c>
       <c r="N39" t="n">
-        <v>0.6958</v>
+        <v>0.6996</v>
       </c>
       <c r="O39" t="n">
-        <v>0.7399</v>
+        <v>0.7439</v>
       </c>
       <c r="P39" t="n">
-        <v>0.7828000000000001</v>
+        <v>0.7871</v>
       </c>
       <c r="Q39" t="n">
-        <v>0.8233</v>
+        <v>0.828</v>
       </c>
       <c r="R39" t="n">
-        <v>0.8648</v>
+        <v>0.8697</v>
       </c>
       <c r="S39" t="n">
-        <v>0.9092</v>
+        <v>0.9145</v>
       </c>
       <c r="T39" t="n">
-        <v>0.9442</v>
+        <v>0.9497</v>
       </c>
       <c r="U39" t="n">
-        <v>0.9883999999999999</v>
+        <v>0.9942</v>
       </c>
       <c r="V39" t="n">
-        <v>1.0347</v>
+        <v>1.0409</v>
       </c>
       <c r="W39" t="n">
-        <v>1.0708</v>
+        <v>1.0772</v>
       </c>
       <c r="X39" t="n">
-        <v>1.1137</v>
+        <v>1.1204</v>
       </c>
       <c r="Y39" t="n">
-        <v>1.1537</v>
+        <v>1.1607</v>
       </c>
       <c r="Z39" t="n">
-        <v>1.1874</v>
+        <v>1.1946</v>
       </c>
       <c r="AA39" t="n">
-        <v>1.2324</v>
+        <v>1.2399</v>
       </c>
       <c r="AB39" t="n">
-        <v>1.2725</v>
+        <v>1.2804</v>
       </c>
       <c r="AC39" t="n">
-        <v>1.3116</v>
+        <v>1.3197</v>
       </c>
       <c r="AD39" t="n">
-        <v>1.3566</v>
+        <v>1.365</v>
       </c>
       <c r="AE39" t="n">
-        <v>1.3933</v>
+        <v>1.402</v>
       </c>
       <c r="AF39" t="n">
-        <v>1.4318</v>
+        <v>1.4407</v>
       </c>
       <c r="AG39" t="n">
-        <v>1.4634</v>
+        <v>1.4725</v>
       </c>
       <c r="AH39" t="n">
-        <v>1.5099</v>
+        <v>1.5194</v>
       </c>
       <c r="AI39" t="n">
-        <v>1.552</v>
+        <v>1.5618</v>
       </c>
       <c r="AJ39" t="n">
-        <v>1.5839</v>
+        <v>1.5939</v>
       </c>
       <c r="AK39" t="n">
-        <v>1.629</v>
+        <v>1.6393</v>
       </c>
       <c r="AL39" t="n">
-        <v>1.6709</v>
+        <v>1.6814</v>
       </c>
     </row>
     <row r="40">
@@ -1406,112 +1406,112 @@
         <v>0.1688</v>
       </c>
       <c r="C40" t="n">
-        <v>0.2045</v>
+        <v>0.2051</v>
       </c>
       <c r="D40" t="n">
-        <v>0.2494</v>
+        <v>0.2506</v>
       </c>
       <c r="E40" t="n">
-        <v>0.2918</v>
+        <v>0.2937</v>
       </c>
       <c r="F40" t="n">
-        <v>0.3361</v>
+        <v>0.3386</v>
       </c>
       <c r="G40" t="n">
-        <v>0.3769</v>
+        <v>0.3801</v>
       </c>
       <c r="H40" t="n">
-        <v>0.4213</v>
+        <v>0.4251</v>
       </c>
       <c r="I40" t="n">
-        <v>0.4614</v>
+        <v>0.4659</v>
       </c>
       <c r="J40" t="n">
-        <v>0.5042</v>
+        <v>0.5093</v>
       </c>
       <c r="K40" t="n">
-        <v>0.5429</v>
+        <v>0.5485</v>
       </c>
       <c r="L40" t="n">
-        <v>0.5863</v>
+        <v>0.5927</v>
       </c>
       <c r="M40" t="n">
-        <v>0.6276</v>
+        <v>0.6346000000000001</v>
       </c>
       <c r="N40" t="n">
-        <v>0.6702</v>
+        <v>0.6778</v>
       </c>
       <c r="O40" t="n">
-        <v>0.7109</v>
+        <v>0.7191</v>
       </c>
       <c r="P40" t="n">
-        <v>0.7516</v>
+        <v>0.7604</v>
       </c>
       <c r="Q40" t="n">
-        <v>0.7922</v>
+        <v>0.8016</v>
       </c>
       <c r="R40" t="n">
-        <v>0.8358</v>
+        <v>0.8459</v>
       </c>
       <c r="S40" t="n">
-        <v>0.871</v>
+        <v>0.8816000000000001</v>
       </c>
       <c r="T40" t="n">
-        <v>0.9159</v>
+        <v>0.9271</v>
       </c>
       <c r="U40" t="n">
-        <v>0.9540999999999999</v>
+        <v>0.9659</v>
       </c>
       <c r="V40" t="n">
-        <v>0.9972</v>
+        <v>1.0096</v>
       </c>
       <c r="W40" t="n">
-        <v>1.0296</v>
+        <v>1.0425</v>
       </c>
       <c r="X40" t="n">
-        <v>1.0683</v>
+        <v>1.0818</v>
       </c>
       <c r="Y40" t="n">
-        <v>1.1109</v>
+        <v>1.125</v>
       </c>
       <c r="Z40" t="n">
-        <v>1.1557</v>
+        <v>1.1705</v>
       </c>
       <c r="AA40" t="n">
-        <v>1.1877</v>
+        <v>1.2029</v>
       </c>
       <c r="AB40" t="n">
-        <v>1.2359</v>
+        <v>1.2518</v>
       </c>
       <c r="AC40" t="n">
-        <v>1.2669</v>
+        <v>1.2832</v>
       </c>
       <c r="AD40" t="n">
-        <v>1.314</v>
+        <v>1.3311</v>
       </c>
       <c r="AE40" t="n">
-        <v>1.3551</v>
+        <v>1.3727</v>
       </c>
       <c r="AF40" t="n">
-        <v>1.3872</v>
+        <v>1.4053</v>
       </c>
       <c r="AG40" t="n">
-        <v>1.4292</v>
+        <v>1.448</v>
       </c>
       <c r="AH40" t="n">
-        <v>1.4669</v>
+        <v>1.4862</v>
       </c>
       <c r="AI40" t="n">
-        <v>1.5002</v>
+        <v>1.5199</v>
       </c>
       <c r="AJ40" t="n">
-        <v>1.5421</v>
+        <v>1.5625</v>
       </c>
       <c r="AK40" t="n">
-        <v>1.5792</v>
+        <v>1.6001</v>
       </c>
       <c r="AL40" t="n">
-        <v>1.6277</v>
+        <v>1.6494</v>
       </c>
     </row>
     <row r="41">
@@ -1524,112 +1524,112 @@
         <v>0.1776</v>
       </c>
       <c r="C41" t="n">
-        <v>0.2209</v>
+        <v>0.2221</v>
       </c>
       <c r="D41" t="n">
-        <v>0.2639</v>
+        <v>0.2665</v>
       </c>
       <c r="E41" t="n">
-        <v>0.307</v>
+        <v>0.3109</v>
       </c>
       <c r="F41" t="n">
-        <v>0.3525</v>
+        <v>0.3578</v>
       </c>
       <c r="G41" t="n">
-        <v>0.3951</v>
+        <v>0.4017</v>
       </c>
       <c r="H41" t="n">
-        <v>0.4397</v>
+        <v>0.4477</v>
       </c>
       <c r="I41" t="n">
-        <v>0.4828</v>
+        <v>0.492</v>
       </c>
       <c r="J41" t="n">
-        <v>0.5292</v>
+        <v>0.5397999999999999</v>
       </c>
       <c r="K41" t="n">
-        <v>0.572</v>
+        <v>0.5839</v>
       </c>
       <c r="L41" t="n">
-        <v>0.612</v>
+        <v>0.6251</v>
       </c>
       <c r="M41" t="n">
-        <v>0.6572</v>
+        <v>0.6717</v>
       </c>
       <c r="N41" t="n">
-        <v>0.6958</v>
+        <v>0.7116</v>
       </c>
       <c r="O41" t="n">
-        <v>0.744</v>
+        <v>0.7612</v>
       </c>
       <c r="P41" t="n">
-        <v>0.7846</v>
+        <v>0.803</v>
       </c>
       <c r="Q41" t="n">
-        <v>0.8285</v>
+        <v>0.8482</v>
       </c>
       <c r="R41" t="n">
-        <v>0.8647</v>
+        <v>0.8856000000000001</v>
       </c>
       <c r="S41" t="n">
-        <v>0.9093</v>
+        <v>0.9315</v>
       </c>
       <c r="T41" t="n">
-        <v>0.9489</v>
+        <v>0.9723000000000001</v>
       </c>
       <c r="U41" t="n">
-        <v>0.991</v>
+        <v>1.0157</v>
       </c>
       <c r="V41" t="n">
-        <v>1.0368</v>
+        <v>1.063</v>
       </c>
       <c r="W41" t="n">
-        <v>1.0799</v>
+        <v>1.1074</v>
       </c>
       <c r="X41" t="n">
-        <v>1.1166</v>
+        <v>1.1451</v>
       </c>
       <c r="Y41" t="n">
-        <v>1.156</v>
+        <v>1.1858</v>
       </c>
       <c r="Z41" t="n">
-        <v>1.1973</v>
+        <v>1.2284</v>
       </c>
       <c r="AA41" t="n">
-        <v>1.2416</v>
+        <v>1.274</v>
       </c>
       <c r="AB41" t="n">
-        <v>1.2799</v>
+        <v>1.3134</v>
       </c>
       <c r="AC41" t="n">
-        <v>1.3208</v>
+        <v>1.3556</v>
       </c>
       <c r="AD41" t="n">
-        <v>1.357</v>
+        <v>1.393</v>
       </c>
       <c r="AE41" t="n">
-        <v>1.4038</v>
+        <v>1.4412</v>
       </c>
       <c r="AF41" t="n">
-        <v>1.4422</v>
+        <v>1.4807</v>
       </c>
       <c r="AG41" t="n">
-        <v>1.4904</v>
+        <v>1.5304</v>
       </c>
       <c r="AH41" t="n">
-        <v>1.5276</v>
+        <v>1.5688</v>
       </c>
       <c r="AI41" t="n">
-        <v>1.5552</v>
+        <v>1.5972</v>
       </c>
       <c r="AJ41" t="n">
-        <v>1.5952</v>
+        <v>1.6385</v>
       </c>
       <c r="AK41" t="n">
-        <v>1.6312</v>
+        <v>1.6756</v>
       </c>
       <c r="AL41" t="n">
-        <v>1.6858</v>
+        <v>1.7318</v>
       </c>
     </row>
     <row r="42">
@@ -1642,112 +1642,112 @@
         <v>0.1691</v>
       </c>
       <c r="C42" t="n">
-        <v>0.2063</v>
+        <v>0.2085</v>
       </c>
       <c r="D42" t="n">
-        <v>0.2468</v>
+        <v>0.2515</v>
       </c>
       <c r="E42" t="n">
-        <v>0.291</v>
+        <v>0.2983</v>
       </c>
       <c r="F42" t="n">
-        <v>0.332</v>
+        <v>0.3417</v>
       </c>
       <c r="G42" t="n">
-        <v>0.3735</v>
+        <v>0.3857</v>
       </c>
       <c r="H42" t="n">
-        <v>0.4142</v>
+        <v>0.429</v>
       </c>
       <c r="I42" t="n">
-        <v>0.4542</v>
+        <v>0.4713</v>
       </c>
       <c r="J42" t="n">
-        <v>0.4987</v>
+        <v>0.5185</v>
       </c>
       <c r="K42" t="n">
-        <v>0.5406</v>
+        <v>0.5629999999999999</v>
       </c>
       <c r="L42" t="n">
-        <v>0.5773</v>
+        <v>0.602</v>
       </c>
       <c r="M42" t="n">
-        <v>0.6183999999999999</v>
+        <v>0.6456</v>
       </c>
       <c r="N42" t="n">
-        <v>0.6592</v>
+        <v>0.6889</v>
       </c>
       <c r="O42" t="n">
-        <v>0.6979</v>
+        <v>0.7301</v>
       </c>
       <c r="P42" t="n">
-        <v>0.7372</v>
+        <v>0.7717000000000001</v>
       </c>
       <c r="Q42" t="n">
-        <v>0.7811</v>
+        <v>0.8182</v>
       </c>
       <c r="R42" t="n">
-        <v>0.8179</v>
+        <v>0.8573</v>
       </c>
       <c r="S42" t="n">
-        <v>0.8593</v>
+        <v>0.9013</v>
       </c>
       <c r="T42" t="n">
-        <v>0.8922</v>
+        <v>0.9365</v>
       </c>
       <c r="U42" t="n">
-        <v>0.9316</v>
+        <v>0.9782999999999999</v>
       </c>
       <c r="V42" t="n">
-        <v>0.9775</v>
+        <v>1.0271</v>
       </c>
       <c r="W42" t="n">
-        <v>1.0173</v>
+        <v>1.0694</v>
       </c>
       <c r="X42" t="n">
-        <v>1.0486</v>
+        <v>1.1028</v>
       </c>
       <c r="Y42" t="n">
-        <v>1.0872</v>
+        <v>1.1438</v>
       </c>
       <c r="Z42" t="n">
-        <v>1.1279</v>
+        <v>1.1872</v>
       </c>
       <c r="AA42" t="n">
-        <v>1.1677</v>
+        <v>1.2295</v>
       </c>
       <c r="AB42" t="n">
-        <v>1.203</v>
+        <v>1.2671</v>
       </c>
       <c r="AC42" t="n">
-        <v>1.2386</v>
+        <v>1.305</v>
       </c>
       <c r="AD42" t="n">
-        <v>1.2784</v>
+        <v>1.3474</v>
       </c>
       <c r="AE42" t="n">
-        <v>1.3172</v>
+        <v>1.3888</v>
       </c>
       <c r="AF42" t="n">
-        <v>1.3564</v>
+        <v>1.4306</v>
       </c>
       <c r="AG42" t="n">
-        <v>1.3973</v>
+        <v>1.4741</v>
       </c>
       <c r="AH42" t="n">
-        <v>1.4273</v>
+        <v>1.5061</v>
       </c>
       <c r="AI42" t="n">
-        <v>1.4606</v>
+        <v>1.5416</v>
       </c>
       <c r="AJ42" t="n">
-        <v>1.4969</v>
+        <v>1.5804</v>
       </c>
       <c r="AK42" t="n">
-        <v>1.539</v>
+        <v>1.6254</v>
       </c>
       <c r="AL42" t="n">
-        <v>1.5736</v>
+        <v>1.6623</v>
       </c>
     </row>
     <row r="43">
@@ -1760,112 +1760,112 @@
         <v>0.1546</v>
       </c>
       <c r="C43" t="n">
-        <v>0.1879</v>
+        <v>0.1916</v>
       </c>
       <c r="D43" t="n">
-        <v>0.2264</v>
+        <v>0.2343</v>
       </c>
       <c r="E43" t="n">
-        <v>0.2628</v>
+        <v>0.2749</v>
       </c>
       <c r="F43" t="n">
-        <v>0.2981</v>
+        <v>0.3144</v>
       </c>
       <c r="G43" t="n">
-        <v>0.3358</v>
+        <v>0.3564</v>
       </c>
       <c r="H43" t="n">
-        <v>0.3745</v>
+        <v>0.3994</v>
       </c>
       <c r="I43" t="n">
-        <v>0.407</v>
+        <v>0.4361</v>
       </c>
       <c r="J43" t="n">
-        <v>0.4405</v>
+        <v>0.4737</v>
       </c>
       <c r="K43" t="n">
-        <v>0.4772</v>
+        <v>0.5147</v>
       </c>
       <c r="L43" t="n">
-        <v>0.5133</v>
+        <v>0.5548999999999999</v>
       </c>
       <c r="M43" t="n">
-        <v>0.5481</v>
+        <v>0.5939</v>
       </c>
       <c r="N43" t="n">
-        <v>0.5827</v>
+        <v>0.6328</v>
       </c>
       <c r="O43" t="n">
-        <v>0.6205000000000001</v>
+        <v>0.6752</v>
       </c>
       <c r="P43" t="n">
-        <v>0.6539</v>
+        <v>0.7126</v>
       </c>
       <c r="Q43" t="n">
-        <v>0.6884</v>
+        <v>0.7516</v>
       </c>
       <c r="R43" t="n">
-        <v>0.7223000000000001</v>
+        <v>0.7896</v>
       </c>
       <c r="S43" t="n">
-        <v>0.7547</v>
+        <v>0.8260999999999999</v>
       </c>
       <c r="T43" t="n">
-        <v>0.792</v>
+        <v>0.868</v>
       </c>
       <c r="U43" t="n">
-        <v>0.8193</v>
+        <v>0.899</v>
       </c>
       <c r="V43" t="n">
-        <v>0.8542999999999999</v>
+        <v>0.9387</v>
       </c>
       <c r="W43" t="n">
-        <v>0.8895</v>
+        <v>0.9782</v>
       </c>
       <c r="X43" t="n">
-        <v>0.9171</v>
+        <v>1.0095</v>
       </c>
       <c r="Y43" t="n">
-        <v>0.9519</v>
+        <v>1.0488</v>
       </c>
       <c r="Z43" t="n">
-        <v>0.9818</v>
+        <v>1.0829</v>
       </c>
       <c r="AA43" t="n">
-        <v>1.0193</v>
+        <v>1.1251</v>
       </c>
       <c r="AB43" t="n">
-        <v>1.0507</v>
+        <v>1.1609</v>
       </c>
       <c r="AC43" t="n">
-        <v>1.0785</v>
+        <v>1.1925</v>
       </c>
       <c r="AD43" t="n">
-        <v>1.1117</v>
+        <v>1.2302</v>
       </c>
       <c r="AE43" t="n">
-        <v>1.1457</v>
+        <v>1.2687</v>
       </c>
       <c r="AF43" t="n">
-        <v>1.1717</v>
+        <v>1.2987</v>
       </c>
       <c r="AG43" t="n">
-        <v>1.2102</v>
+        <v>1.342</v>
       </c>
       <c r="AH43" t="n">
-        <v>1.2406</v>
+        <v>1.3769</v>
       </c>
       <c r="AI43" t="n">
-        <v>1.262</v>
+        <v>1.4016</v>
       </c>
       <c r="AJ43" t="n">
-        <v>1.2926</v>
+        <v>1.4362</v>
       </c>
       <c r="AK43" t="n">
-        <v>1.3242</v>
+        <v>1.4723</v>
       </c>
       <c r="AL43" t="n">
-        <v>1.3541</v>
+        <v>1.5066</v>
       </c>
     </row>
     <row r="44">
@@ -1878,112 +1878,112 @@
         <v>0.1622</v>
       </c>
       <c r="C44" t="n">
-        <v>0.1904</v>
+        <v>0.1963</v>
       </c>
       <c r="D44" t="n">
-        <v>0.2234</v>
+        <v>0.236</v>
       </c>
       <c r="E44" t="n">
-        <v>0.2551</v>
+        <v>0.2745</v>
       </c>
       <c r="F44" t="n">
-        <v>0.288</v>
+        <v>0.314</v>
       </c>
       <c r="G44" t="n">
-        <v>0.3155</v>
+        <v>0.3481</v>
       </c>
       <c r="H44" t="n">
-        <v>0.3498</v>
+        <v>0.3891</v>
       </c>
       <c r="I44" t="n">
-        <v>0.3804</v>
+        <v>0.4264</v>
       </c>
       <c r="J44" t="n">
-        <v>0.4101</v>
+        <v>0.4626</v>
       </c>
       <c r="K44" t="n">
-        <v>0.4415</v>
+        <v>0.5004999999999999</v>
       </c>
       <c r="L44" t="n">
-        <v>0.4732</v>
+        <v>0.5389</v>
       </c>
       <c r="M44" t="n">
-        <v>0.5032</v>
+        <v>0.5750999999999999</v>
       </c>
       <c r="N44" t="n">
-        <v>0.5285</v>
+        <v>0.6066</v>
       </c>
       <c r="O44" t="n">
-        <v>0.555</v>
+        <v>0.6393</v>
       </c>
       <c r="P44" t="n">
-        <v>0.5848</v>
+        <v>0.6756</v>
       </c>
       <c r="Q44" t="n">
-        <v>0.6124000000000001</v>
+        <v>0.7095</v>
       </c>
       <c r="R44" t="n">
-        <v>0.6409</v>
+        <v>0.7445000000000001</v>
       </c>
       <c r="S44" t="n">
-        <v>0.6672</v>
+        <v>0.7764</v>
       </c>
       <c r="T44" t="n">
-        <v>0.6964</v>
+        <v>0.8116</v>
       </c>
       <c r="U44" t="n">
-        <v>0.7212</v>
+        <v>0.8425</v>
       </c>
       <c r="V44" t="n">
-        <v>0.7485000000000001</v>
+        <v>0.8754999999999999</v>
       </c>
       <c r="W44" t="n">
-        <v>0.7723</v>
+        <v>0.9048</v>
       </c>
       <c r="X44" t="n">
-        <v>0.7937</v>
+        <v>0.9308999999999999</v>
       </c>
       <c r="Y44" t="n">
-        <v>0.8224</v>
+        <v>0.9657</v>
       </c>
       <c r="Z44" t="n">
-        <v>0.8493000000000001</v>
+        <v>0.998</v>
       </c>
       <c r="AA44" t="n">
-        <v>0.8685</v>
+        <v>1.0219</v>
       </c>
       <c r="AB44" t="n">
-        <v>0.8993</v>
+        <v>1.0585</v>
       </c>
       <c r="AC44" t="n">
-        <v>0.9094</v>
+        <v>1.0708</v>
       </c>
       <c r="AD44" t="n">
-        <v>0.9418</v>
+        <v>1.1099</v>
       </c>
       <c r="AE44" t="n">
-        <v>0.9563</v>
+        <v>1.127</v>
       </c>
       <c r="AF44" t="n">
-        <v>0.9806</v>
+        <v>1.1556</v>
       </c>
       <c r="AG44" t="n">
-        <v>1.0033</v>
+        <v>1.1817</v>
       </c>
       <c r="AH44" t="n">
-        <v>1.0258</v>
+        <v>1.2084</v>
       </c>
       <c r="AI44" t="n">
-        <v>1.0416</v>
+        <v>1.226</v>
       </c>
       <c r="AJ44" t="n">
-        <v>1.0607</v>
+        <v>1.248</v>
       </c>
       <c r="AK44" t="n">
-        <v>1.0839</v>
+        <v>1.2742</v>
       </c>
       <c r="AL44" t="n">
-        <v>1.099</v>
+        <v>1.2905</v>
       </c>
     </row>
     <row r="45">
@@ -1996,112 +1996,112 @@
         <v>0.1582</v>
       </c>
       <c r="C45" t="n">
-        <v>0.1666</v>
+        <v>0.1682</v>
       </c>
       <c r="D45" t="n">
-        <v>0.176</v>
+        <v>0.1816</v>
       </c>
       <c r="E45" t="n">
-        <v>0.1915</v>
+        <v>0.2027</v>
       </c>
       <c r="F45" t="n">
-        <v>0.2126</v>
+        <v>0.2303</v>
       </c>
       <c r="G45" t="n">
-        <v>0.235</v>
+        <v>0.26</v>
       </c>
       <c r="H45" t="n">
-        <v>0.2551</v>
+        <v>0.2874</v>
       </c>
       <c r="I45" t="n">
-        <v>0.2779</v>
+        <v>0.3177</v>
       </c>
       <c r="J45" t="n">
-        <v>0.3003</v>
+        <v>0.3475</v>
       </c>
       <c r="K45" t="n">
-        <v>0.3208</v>
+        <v>0.3754</v>
       </c>
       <c r="L45" t="n">
-        <v>0.3445</v>
+        <v>0.4062</v>
       </c>
       <c r="M45" t="n">
-        <v>0.3653</v>
+        <v>0.434</v>
       </c>
       <c r="N45" t="n">
-        <v>0.3885</v>
+        <v>0.4643</v>
       </c>
       <c r="O45" t="n">
-        <v>0.409</v>
+        <v>0.491</v>
       </c>
       <c r="P45" t="n">
-        <v>0.4265</v>
+        <v>0.5141</v>
       </c>
       <c r="Q45" t="n">
-        <v>0.4458</v>
+        <v>0.539</v>
       </c>
       <c r="R45" t="n">
-        <v>0.4614</v>
+        <v>0.5595</v>
       </c>
       <c r="S45" t="n">
-        <v>0.4849</v>
+        <v>0.5884</v>
       </c>
       <c r="T45" t="n">
-        <v>0.5006</v>
+        <v>0.6078</v>
       </c>
       <c r="U45" t="n">
-        <v>0.5204</v>
+        <v>0.6319</v>
       </c>
       <c r="V45" t="n">
-        <v>0.5362</v>
+        <v>0.6506</v>
       </c>
       <c r="W45" t="n">
-        <v>0.553</v>
+        <v>0.6706</v>
       </c>
       <c r="X45" t="n">
-        <v>0.5675</v>
+        <v>0.6874</v>
       </c>
       <c r="Y45" t="n">
-        <v>0.5822000000000001</v>
+        <v>0.7032</v>
       </c>
       <c r="Z45" t="n">
-        <v>0.5983000000000001</v>
+        <v>0.7213000000000001</v>
       </c>
       <c r="AA45" t="n">
-        <v>0.609</v>
+        <v>0.7319</v>
       </c>
       <c r="AB45" t="n">
-        <v>0.6244</v>
+        <v>0.7481</v>
       </c>
       <c r="AC45" t="n">
-        <v>0.6347</v>
+        <v>0.7576000000000001</v>
       </c>
       <c r="AD45" t="n">
-        <v>0.6495</v>
+        <v>0.7723</v>
       </c>
       <c r="AE45" t="n">
-        <v>0.6643</v>
+        <v>0.786</v>
       </c>
       <c r="AF45" t="n">
-        <v>0.672</v>
+        <v>0.7915</v>
       </c>
       <c r="AG45" t="n">
-        <v>0.6843</v>
+        <v>0.8025</v>
       </c>
       <c r="AH45" t="n">
-        <v>0.6962</v>
+        <v>0.8122</v>
       </c>
       <c r="AI45" t="n">
-        <v>0.7036</v>
+        <v>0.8165</v>
       </c>
       <c r="AJ45" t="n">
-        <v>0.7131</v>
+        <v>0.8232</v>
       </c>
       <c r="AK45" t="n">
-        <v>0.7234</v>
+        <v>0.8312</v>
       </c>
       <c r="AL45" t="n">
-        <v>0.7334000000000001</v>
+        <v>0.8373</v>
       </c>
     </row>
     <row r="46">
@@ -2114,112 +2114,112 @@
         <v>0.1695</v>
       </c>
       <c r="C46" t="n">
-        <v>0.1824</v>
+        <v>0.1887</v>
       </c>
       <c r="D46" t="n">
-        <v>0.1962</v>
+        <v>0.2095</v>
       </c>
       <c r="E46" t="n">
-        <v>0.2093</v>
+        <v>0.229</v>
       </c>
       <c r="F46" t="n">
-        <v>0.2217</v>
+        <v>0.2477</v>
       </c>
       <c r="G46" t="n">
-        <v>0.2371</v>
+        <v>0.2691</v>
       </c>
       <c r="H46" t="n">
-        <v>0.2477</v>
+        <v>0.2851</v>
       </c>
       <c r="I46" t="n">
-        <v>0.2608</v>
+        <v>0.3035</v>
       </c>
       <c r="J46" t="n">
-        <v>0.2734</v>
+        <v>0.3205</v>
       </c>
       <c r="K46" t="n">
-        <v>0.2829</v>
+        <v>0.3344</v>
       </c>
       <c r="L46" t="n">
-        <v>0.2936</v>
+        <v>0.3487</v>
       </c>
       <c r="M46" t="n">
-        <v>0.3047</v>
+        <v>0.3633</v>
       </c>
       <c r="N46" t="n">
-        <v>0.3151</v>
+        <v>0.377</v>
       </c>
       <c r="O46" t="n">
-        <v>0.324</v>
+        <v>0.3884</v>
       </c>
       <c r="P46" t="n">
-        <v>0.3308</v>
+        <v>0.3968</v>
       </c>
       <c r="Q46" t="n">
-        <v>0.3444</v>
+        <v>0.4129</v>
       </c>
       <c r="R46" t="n">
-        <v>0.3518</v>
+        <v>0.4219</v>
       </c>
       <c r="S46" t="n">
-        <v>0.3601</v>
+        <v>0.4309</v>
       </c>
       <c r="T46" t="n">
-        <v>0.3693</v>
+        <v>0.441</v>
       </c>
       <c r="U46" t="n">
-        <v>0.3773</v>
+        <v>0.4495</v>
       </c>
       <c r="V46" t="n">
-        <v>0.3835</v>
+        <v>0.4552</v>
       </c>
       <c r="W46" t="n">
-        <v>0.3876</v>
+        <v>0.459</v>
       </c>
       <c r="X46" t="n">
-        <v>0.3995</v>
+        <v>0.4711</v>
       </c>
       <c r="Y46" t="n">
-        <v>0.404</v>
+        <v>0.4747</v>
       </c>
       <c r="Z46" t="n">
-        <v>0.4108</v>
+        <v>0.4806</v>
       </c>
       <c r="AA46" t="n">
-        <v>0.4153</v>
+        <v>0.4841</v>
       </c>
       <c r="AB46" t="n">
-        <v>0.4218</v>
+        <v>0.4887</v>
       </c>
       <c r="AC46" t="n">
-        <v>0.4248</v>
+        <v>0.4904</v>
       </c>
       <c r="AD46" t="n">
-        <v>0.4321</v>
+        <v>0.4963</v>
       </c>
       <c r="AE46" t="n">
-        <v>0.4406</v>
+        <v>0.5032</v>
       </c>
       <c r="AF46" t="n">
-        <v>0.4448</v>
+        <v>0.506</v>
       </c>
       <c r="AG46" t="n">
-        <v>0.4464</v>
+        <v>0.5051</v>
       </c>
       <c r="AH46" t="n">
-        <v>0.4502</v>
+        <v>0.5072</v>
       </c>
       <c r="AI46" t="n">
-        <v>0.4547</v>
+        <v>0.5097</v>
       </c>
       <c r="AJ46" t="n">
-        <v>0.4617</v>
+        <v>0.5152</v>
       </c>
       <c r="AK46" t="n">
-        <v>0.4641</v>
+        <v>0.5153</v>
       </c>
       <c r="AL46" t="n">
-        <v>0.4667</v>
+        <v>0.5161</v>
       </c>
     </row>
     <row r="47">
@@ -2232,112 +2232,112 @@
         <v>0.1679</v>
       </c>
       <c r="C47" t="n">
-        <v>0.1747</v>
+        <v>0.1802</v>
       </c>
       <c r="D47" t="n">
-        <v>0.1825</v>
+        <v>0.1938</v>
       </c>
       <c r="E47" t="n">
-        <v>0.1944</v>
+        <v>0.2108</v>
       </c>
       <c r="F47" t="n">
-        <v>0.2018</v>
+        <v>0.2228</v>
       </c>
       <c r="G47" t="n">
-        <v>0.2095</v>
+        <v>0.2345</v>
       </c>
       <c r="H47" t="n">
-        <v>0.2175</v>
+        <v>0.2458</v>
       </c>
       <c r="I47" t="n">
-        <v>0.2257</v>
+        <v>0.257</v>
       </c>
       <c r="J47" t="n">
-        <v>0.2318</v>
+        <v>0.2655</v>
       </c>
       <c r="K47" t="n">
-        <v>0.2392</v>
+        <v>0.2749</v>
       </c>
       <c r="L47" t="n">
-        <v>0.245</v>
+        <v>0.2822</v>
       </c>
       <c r="M47" t="n">
-        <v>0.2509</v>
+        <v>0.2892</v>
       </c>
       <c r="N47" t="n">
-        <v>0.258</v>
+        <v>0.2972</v>
       </c>
       <c r="O47" t="n">
-        <v>0.2623</v>
+        <v>0.3018</v>
       </c>
       <c r="P47" t="n">
-        <v>0.2659</v>
+        <v>0.3055</v>
       </c>
       <c r="Q47" t="n">
-        <v>0.2731</v>
+        <v>0.3127</v>
       </c>
       <c r="R47" t="n">
-        <v>0.2742</v>
+        <v>0.3131</v>
       </c>
       <c r="S47" t="n">
-        <v>0.2809</v>
+        <v>0.3196</v>
       </c>
       <c r="T47" t="n">
-        <v>0.2846</v>
+        <v>0.3224</v>
       </c>
       <c r="U47" t="n">
-        <v>0.2898</v>
+        <v>0.3269</v>
       </c>
       <c r="V47" t="n">
-        <v>0.2938</v>
+        <v>0.3298</v>
       </c>
       <c r="W47" t="n">
-        <v>0.2955</v>
+        <v>0.3306</v>
       </c>
       <c r="X47" t="n">
-        <v>0.3005</v>
+        <v>0.3344</v>
       </c>
       <c r="Y47" t="n">
-        <v>0.3023</v>
+        <v>0.3349</v>
       </c>
       <c r="Z47" t="n">
-        <v>0.3061</v>
+        <v>0.3375</v>
       </c>
       <c r="AA47" t="n">
-        <v>0.3086</v>
+        <v>0.3386</v>
       </c>
       <c r="AB47" t="n">
-        <v>0.3105</v>
+        <v>0.3392</v>
       </c>
       <c r="AC47" t="n">
-        <v>0.3149</v>
+        <v>0.3426</v>
       </c>
       <c r="AD47" t="n">
-        <v>0.3169</v>
+        <v>0.3432</v>
       </c>
       <c r="AE47" t="n">
-        <v>0.3171</v>
+        <v>0.342</v>
       </c>
       <c r="AF47" t="n">
-        <v>0.3184</v>
+        <v>0.3423</v>
       </c>
       <c r="AG47" t="n">
-        <v>0.3197</v>
+        <v>0.3423</v>
       </c>
       <c r="AH47" t="n">
-        <v>0.3243</v>
+        <v>0.3459</v>
       </c>
       <c r="AI47" t="n">
-        <v>0.3267</v>
+        <v>0.3472</v>
       </c>
       <c r="AJ47" t="n">
-        <v>0.3279</v>
+        <v>0.3472</v>
       </c>
       <c r="AK47" t="n">
-        <v>0.328</v>
+        <v>0.3463</v>
       </c>
       <c r="AL47" t="n">
-        <v>0.3286</v>
+        <v>0.3459</v>
       </c>
     </row>
     <row r="48">
@@ -2471,109 +2471,109 @@
         <v>0.2209</v>
       </c>
       <c r="D49" t="n">
-        <v>0.2596</v>
+        <v>0.2597</v>
       </c>
       <c r="E49" t="n">
-        <v>0.2985</v>
+        <v>0.2986</v>
       </c>
       <c r="F49" t="n">
-        <v>0.3357</v>
+        <v>0.336</v>
       </c>
       <c r="G49" t="n">
-        <v>0.3726</v>
+        <v>0.3729</v>
       </c>
       <c r="H49" t="n">
-        <v>0.415</v>
+        <v>0.4153</v>
       </c>
       <c r="I49" t="n">
-        <v>0.4507</v>
+        <v>0.4511</v>
       </c>
       <c r="J49" t="n">
-        <v>0.4902</v>
+        <v>0.4907</v>
       </c>
       <c r="K49" t="n">
-        <v>0.5256</v>
+        <v>0.5261</v>
       </c>
       <c r="L49" t="n">
-        <v>0.5638</v>
+        <v>0.5644</v>
       </c>
       <c r="M49" t="n">
-        <v>0.6022</v>
+        <v>0.6029</v>
       </c>
       <c r="N49" t="n">
-        <v>0.6408</v>
+        <v>0.6415</v>
       </c>
       <c r="O49" t="n">
-        <v>0.675</v>
+        <v>0.6758</v>
       </c>
       <c r="P49" t="n">
-        <v>0.7148</v>
+        <v>0.7156</v>
       </c>
       <c r="Q49" t="n">
-        <v>0.7524999999999999</v>
+        <v>0.7534</v>
       </c>
       <c r="R49" t="n">
-        <v>0.7914</v>
+        <v>0.7924</v>
       </c>
       <c r="S49" t="n">
-        <v>0.8246</v>
+        <v>0.8256</v>
       </c>
       <c r="T49" t="n">
-        <v>0.8589</v>
+        <v>0.8599</v>
       </c>
       <c r="U49" t="n">
-        <v>0.8985</v>
+        <v>0.8996</v>
       </c>
       <c r="V49" t="n">
-        <v>0.931</v>
+        <v>0.9322</v>
       </c>
       <c r="W49" t="n">
-        <v>0.9734</v>
+        <v>0.9746</v>
       </c>
       <c r="X49" t="n">
-        <v>1.0057</v>
+        <v>1.007</v>
       </c>
       <c r="Y49" t="n">
-        <v>1.0451</v>
+        <v>1.0464</v>
       </c>
       <c r="Z49" t="n">
-        <v>1.0807</v>
+        <v>1.082</v>
       </c>
       <c r="AA49" t="n">
-        <v>1.1163</v>
+        <v>1.1178</v>
       </c>
       <c r="AB49" t="n">
-        <v>1.1539</v>
+        <v>1.1554</v>
       </c>
       <c r="AC49" t="n">
-        <v>1.1917</v>
+        <v>1.1933</v>
       </c>
       <c r="AD49" t="n">
-        <v>1.224</v>
+        <v>1.2256</v>
       </c>
       <c r="AE49" t="n">
-        <v>1.2604</v>
+        <v>1.2621</v>
       </c>
       <c r="AF49" t="n">
-        <v>1.2956</v>
+        <v>1.2973</v>
       </c>
       <c r="AG49" t="n">
-        <v>1.3224</v>
+        <v>1.3241</v>
       </c>
       <c r="AH49" t="n">
-        <v>1.3675</v>
+        <v>1.3693</v>
       </c>
       <c r="AI49" t="n">
-        <v>1.4067</v>
+        <v>1.4086</v>
       </c>
       <c r="AJ49" t="n">
-        <v>1.435</v>
+        <v>1.4369</v>
       </c>
       <c r="AK49" t="n">
-        <v>1.4763</v>
+        <v>1.4783</v>
       </c>
       <c r="AL49" t="n">
-        <v>1.5095</v>
+        <v>1.5115</v>
       </c>
     </row>
     <row r="50">
@@ -2586,112 +2586,112 @@
         <v>0.1537</v>
       </c>
       <c r="C50" t="n">
-        <v>0.1933</v>
+        <v>0.1934</v>
       </c>
       <c r="D50" t="n">
-        <v>0.2369</v>
+        <v>0.2372</v>
       </c>
       <c r="E50" t="n">
-        <v>0.2787</v>
+        <v>0.2791</v>
       </c>
       <c r="F50" t="n">
-        <v>0.3196</v>
+        <v>0.3201</v>
       </c>
       <c r="G50" t="n">
-        <v>0.3603</v>
+        <v>0.361</v>
       </c>
       <c r="H50" t="n">
-        <v>0.406</v>
+        <v>0.4069</v>
       </c>
       <c r="I50" t="n">
-        <v>0.4481</v>
+        <v>0.4492</v>
       </c>
       <c r="J50" t="n">
-        <v>0.4905</v>
+        <v>0.4917</v>
       </c>
       <c r="K50" t="n">
-        <v>0.53</v>
+        <v>0.5313</v>
       </c>
       <c r="L50" t="n">
-        <v>0.571</v>
+        <v>0.5725</v>
       </c>
       <c r="M50" t="n">
-        <v>0.6151</v>
+        <v>0.6167</v>
       </c>
       <c r="N50" t="n">
-        <v>0.6556</v>
+        <v>0.6573</v>
       </c>
       <c r="O50" t="n">
-        <v>0.6953</v>
+        <v>0.6972</v>
       </c>
       <c r="P50" t="n">
-        <v>0.737</v>
+        <v>0.739</v>
       </c>
       <c r="Q50" t="n">
-        <v>0.7775</v>
+        <v>0.7796999999999999</v>
       </c>
       <c r="R50" t="n">
-        <v>0.8173</v>
+        <v>0.8196</v>
       </c>
       <c r="S50" t="n">
-        <v>0.8592</v>
+        <v>0.8616</v>
       </c>
       <c r="T50" t="n">
-        <v>0.8982</v>
+        <v>0.9006999999999999</v>
       </c>
       <c r="U50" t="n">
-        <v>0.9308999999999999</v>
+        <v>0.9336</v>
       </c>
       <c r="V50" t="n">
-        <v>0.9751</v>
+        <v>0.9779</v>
       </c>
       <c r="W50" t="n">
-        <v>1.0165</v>
+        <v>1.0194</v>
       </c>
       <c r="X50" t="n">
-        <v>1.0548</v>
+        <v>1.0578</v>
       </c>
       <c r="Y50" t="n">
-        <v>1.0948</v>
+        <v>1.098</v>
       </c>
       <c r="Z50" t="n">
-        <v>1.1388</v>
+        <v>1.1421</v>
       </c>
       <c r="AA50" t="n">
-        <v>1.1781</v>
+        <v>1.1816</v>
       </c>
       <c r="AB50" t="n">
-        <v>1.2141</v>
+        <v>1.2177</v>
       </c>
       <c r="AC50" t="n">
-        <v>1.2572</v>
+        <v>1.2609</v>
       </c>
       <c r="AD50" t="n">
-        <v>1.2938</v>
+        <v>1.2976</v>
       </c>
       <c r="AE50" t="n">
-        <v>1.334</v>
+        <v>1.338</v>
       </c>
       <c r="AF50" t="n">
-        <v>1.3723</v>
+        <v>1.3764</v>
       </c>
       <c r="AG50" t="n">
-        <v>1.4107</v>
+        <v>1.415</v>
       </c>
       <c r="AH50" t="n">
-        <v>1.4449</v>
+        <v>1.4492</v>
       </c>
       <c r="AI50" t="n">
-        <v>1.4853</v>
+        <v>1.4898</v>
       </c>
       <c r="AJ50" t="n">
-        <v>1.5232</v>
+        <v>1.5278</v>
       </c>
       <c r="AK50" t="n">
-        <v>1.5595</v>
+        <v>1.5643</v>
       </c>
       <c r="AL50" t="n">
-        <v>1.5989</v>
+        <v>1.6037</v>
       </c>
     </row>
     <row r="51">
@@ -2704,112 +2704,112 @@
         <v>0.1648</v>
       </c>
       <c r="C51" t="n">
-        <v>0.2051</v>
+        <v>0.2054</v>
       </c>
       <c r="D51" t="n">
-        <v>0.249</v>
+        <v>0.2496</v>
       </c>
       <c r="E51" t="n">
-        <v>0.2944</v>
+        <v>0.2953</v>
       </c>
       <c r="F51" t="n">
-        <v>0.339</v>
+        <v>0.3403</v>
       </c>
       <c r="G51" t="n">
-        <v>0.383</v>
+        <v>0.3846</v>
       </c>
       <c r="H51" t="n">
-        <v>0.4663</v>
+        <v>0.4683</v>
       </c>
       <c r="I51" t="n">
-        <v>0.4753</v>
+        <v>0.4775</v>
       </c>
       <c r="J51" t="n">
-        <v>0.5169</v>
+        <v>0.5195</v>
       </c>
       <c r="K51" t="n">
-        <v>0.5592</v>
+        <v>0.5621</v>
       </c>
       <c r="L51" t="n">
-        <v>0.6069</v>
+        <v>0.6102</v>
       </c>
       <c r="M51" t="n">
-        <v>0.6472</v>
+        <v>0.6508</v>
       </c>
       <c r="N51" t="n">
-        <v>0.6905</v>
+        <v>0.6943</v>
       </c>
       <c r="O51" t="n">
-        <v>0.7331</v>
+        <v>0.7373</v>
       </c>
       <c r="P51" t="n">
-        <v>0.778</v>
+        <v>0.7825</v>
       </c>
       <c r="Q51" t="n">
-        <v>0.8201000000000001</v>
+        <v>0.8249</v>
       </c>
       <c r="R51" t="n">
-        <v>0.8643999999999999</v>
+        <v>0.8695000000000001</v>
       </c>
       <c r="S51" t="n">
-        <v>0.9063</v>
+        <v>0.9117</v>
       </c>
       <c r="T51" t="n">
-        <v>0.9504</v>
+        <v>0.9560999999999999</v>
       </c>
       <c r="U51" t="n">
-        <v>0.9932</v>
+        <v>0.9992</v>
       </c>
       <c r="V51" t="n">
-        <v>1.0298</v>
+        <v>1.0361</v>
       </c>
       <c r="W51" t="n">
-        <v>1.0753</v>
+        <v>1.0819</v>
       </c>
       <c r="X51" t="n">
-        <v>1.1171</v>
+        <v>1.124</v>
       </c>
       <c r="Y51" t="n">
-        <v>1.1585</v>
+        <v>1.1656</v>
       </c>
       <c r="Z51" t="n">
-        <v>1.1999</v>
+        <v>1.2073</v>
       </c>
       <c r="AA51" t="n">
-        <v>1.2421</v>
+        <v>1.2499</v>
       </c>
       <c r="AB51" t="n">
-        <v>1.2833</v>
+        <v>1.2914</v>
       </c>
       <c r="AC51" t="n">
-        <v>1.3243</v>
+        <v>1.3327</v>
       </c>
       <c r="AD51" t="n">
-        <v>1.367</v>
+        <v>1.3756</v>
       </c>
       <c r="AE51" t="n">
-        <v>1.4087</v>
+        <v>1.4176</v>
       </c>
       <c r="AF51" t="n">
-        <v>1.4476</v>
+        <v>1.4568</v>
       </c>
       <c r="AG51" t="n">
-        <v>1.4899</v>
+        <v>1.4994</v>
       </c>
       <c r="AH51" t="n">
-        <v>1.5211</v>
+        <v>1.5308</v>
       </c>
       <c r="AI51" t="n">
-        <v>1.5703</v>
+        <v>1.5803</v>
       </c>
       <c r="AJ51" t="n">
-        <v>1.6169</v>
+        <v>1.6272</v>
       </c>
       <c r="AK51" t="n">
-        <v>1.6482</v>
+        <v>1.6588</v>
       </c>
       <c r="AL51" t="n">
-        <v>1.6872</v>
+        <v>1.6981</v>
       </c>
     </row>
     <row r="52">
@@ -2822,112 +2822,112 @@
         <v>0.1795</v>
       </c>
       <c r="C52" t="n">
-        <v>0.2203</v>
+        <v>0.2209</v>
       </c>
       <c r="D52" t="n">
-        <v>0.2666</v>
+        <v>0.2679</v>
       </c>
       <c r="E52" t="n">
-        <v>0.3125</v>
+        <v>0.3145</v>
       </c>
       <c r="F52" t="n">
-        <v>0.3538</v>
+        <v>0.3565</v>
       </c>
       <c r="G52" t="n">
-        <v>0.4</v>
+        <v>0.4034</v>
       </c>
       <c r="H52" t="n">
-        <v>0.4444</v>
+        <v>0.4484</v>
       </c>
       <c r="I52" t="n">
-        <v>0.4888</v>
+        <v>0.4935</v>
       </c>
       <c r="J52" t="n">
-        <v>0.5331</v>
+        <v>0.5384</v>
       </c>
       <c r="K52" t="n">
-        <v>0.5779</v>
+        <v>0.5839</v>
       </c>
       <c r="L52" t="n">
-        <v>0.6197</v>
+        <v>0.6263</v>
       </c>
       <c r="M52" t="n">
-        <v>0.6647</v>
+        <v>0.672</v>
       </c>
       <c r="N52" t="n">
-        <v>0.703</v>
+        <v>0.7109</v>
       </c>
       <c r="O52" t="n">
-        <v>0.7532</v>
+        <v>0.7618</v>
       </c>
       <c r="P52" t="n">
-        <v>0.7943</v>
+        <v>0.8036</v>
       </c>
       <c r="Q52" t="n">
-        <v>0.8375</v>
+        <v>0.8474</v>
       </c>
       <c r="R52" t="n">
-        <v>0.8861</v>
+        <v>0.8967000000000001</v>
       </c>
       <c r="S52" t="n">
-        <v>0.9226</v>
+        <v>0.9337</v>
       </c>
       <c r="T52" t="n">
-        <v>0.9674</v>
+        <v>0.9792</v>
       </c>
       <c r="U52" t="n">
-        <v>1.0104</v>
+        <v>1.0228</v>
       </c>
       <c r="V52" t="n">
-        <v>1.0475</v>
+        <v>1.0604</v>
       </c>
       <c r="W52" t="n">
-        <v>1.0941</v>
+        <v>1.1078</v>
       </c>
       <c r="X52" t="n">
-        <v>1.133</v>
+        <v>1.1473</v>
       </c>
       <c r="Y52" t="n">
-        <v>1.1793</v>
+        <v>1.1942</v>
       </c>
       <c r="Z52" t="n">
-        <v>1.2231</v>
+        <v>1.2387</v>
       </c>
       <c r="AA52" t="n">
-        <v>1.254</v>
+        <v>1.27</v>
       </c>
       <c r="AB52" t="n">
-        <v>1.309</v>
+        <v>1.3258</v>
       </c>
       <c r="AC52" t="n">
-        <v>1.3437</v>
+        <v>1.361</v>
       </c>
       <c r="AD52" t="n">
-        <v>1.3872</v>
+        <v>1.4052</v>
       </c>
       <c r="AE52" t="n">
-        <v>1.422</v>
+        <v>1.4404</v>
       </c>
       <c r="AF52" t="n">
-        <v>1.4647</v>
+        <v>1.4838</v>
       </c>
       <c r="AG52" t="n">
-        <v>1.5106</v>
+        <v>1.5303</v>
       </c>
       <c r="AH52" t="n">
-        <v>1.5516</v>
+        <v>1.572</v>
       </c>
       <c r="AI52" t="n">
-        <v>1.5862</v>
+        <v>1.6071</v>
       </c>
       <c r="AJ52" t="n">
-        <v>1.6259</v>
+        <v>1.6473</v>
       </c>
       <c r="AK52" t="n">
-        <v>1.6643</v>
+        <v>1.6863</v>
       </c>
       <c r="AL52" t="n">
-        <v>1.7077</v>
+        <v>1.7303</v>
       </c>
     </row>
     <row r="53">
@@ -2940,112 +2940,112 @@
         <v>0.1629</v>
       </c>
       <c r="C53" t="n">
-        <v>0.1682</v>
+        <v>0.1683</v>
       </c>
       <c r="D53" t="n">
-        <v>0.1832</v>
+        <v>0.1838</v>
       </c>
       <c r="E53" t="n">
-        <v>0.2038</v>
+        <v>0.205</v>
       </c>
       <c r="F53" t="n">
-        <v>0.2297</v>
+        <v>0.2318</v>
       </c>
       <c r="G53" t="n">
-        <v>0.2628</v>
+        <v>0.2658</v>
       </c>
       <c r="H53" t="n">
-        <v>0.2946</v>
+        <v>0.2986</v>
       </c>
       <c r="I53" t="n">
-        <v>0.3293</v>
+        <v>0.3343</v>
       </c>
       <c r="J53" t="n">
-        <v>0.3659</v>
+        <v>0.372</v>
       </c>
       <c r="K53" t="n">
-        <v>0.4031</v>
+        <v>0.4103</v>
       </c>
       <c r="L53" t="n">
-        <v>0.4417</v>
+        <v>0.4501</v>
       </c>
       <c r="M53" t="n">
-        <v>0.4807</v>
+        <v>0.4903</v>
       </c>
       <c r="N53" t="n">
-        <v>0.5173</v>
+        <v>0.5281</v>
       </c>
       <c r="O53" t="n">
-        <v>0.5581</v>
+        <v>0.5701000000000001</v>
       </c>
       <c r="P53" t="n">
-        <v>0.5993000000000001</v>
+        <v>0.6125</v>
       </c>
       <c r="Q53" t="n">
-        <v>0.6395</v>
+        <v>0.654</v>
       </c>
       <c r="R53" t="n">
-        <v>0.6791</v>
+        <v>0.6947</v>
       </c>
       <c r="S53" t="n">
-        <v>0.7154</v>
+        <v>0.7322</v>
       </c>
       <c r="T53" t="n">
-        <v>0.7584</v>
+        <v>0.7764</v>
       </c>
       <c r="U53" t="n">
-        <v>0.7991</v>
+        <v>0.8184</v>
       </c>
       <c r="V53" t="n">
-        <v>0.8369</v>
+        <v>0.8573</v>
       </c>
       <c r="W53" t="n">
-        <v>0.8771</v>
+        <v>0.8988</v>
       </c>
       <c r="X53" t="n">
-        <v>0.9183</v>
+        <v>0.9412</v>
       </c>
       <c r="Y53" t="n">
-        <v>0.956</v>
+        <v>0.9801</v>
       </c>
       <c r="Z53" t="n">
-        <v>0.993</v>
+        <v>1.0182</v>
       </c>
       <c r="AA53" t="n">
-        <v>1.0338</v>
+        <v>1.0603</v>
       </c>
       <c r="AB53" t="n">
-        <v>1.0755</v>
+        <v>1.1033</v>
       </c>
       <c r="AC53" t="n">
-        <v>1.1122</v>
+        <v>1.1412</v>
       </c>
       <c r="AD53" t="n">
-        <v>1.1503</v>
+        <v>1.1803</v>
       </c>
       <c r="AE53" t="n">
-        <v>1.1868</v>
+        <v>1.2179</v>
       </c>
       <c r="AF53" t="n">
-        <v>1.2323</v>
+        <v>1.2648</v>
       </c>
       <c r="AG53" t="n">
-        <v>1.2687</v>
+        <v>1.3024</v>
       </c>
       <c r="AH53" t="n">
-        <v>1.3084</v>
+        <v>1.3433</v>
       </c>
       <c r="AI53" t="n">
-        <v>1.3474</v>
+        <v>1.3835</v>
       </c>
       <c r="AJ53" t="n">
-        <v>1.3768</v>
+        <v>1.4139</v>
       </c>
       <c r="AK53" t="n">
-        <v>1.4229</v>
+        <v>1.4613</v>
       </c>
       <c r="AL53" t="n">
-        <v>1.4528</v>
+        <v>1.4921</v>
       </c>
     </row>
     <row r="54">
@@ -3058,112 +3058,112 @@
         <v>0.1803</v>
       </c>
       <c r="C54" t="n">
-        <v>0.2157</v>
+        <v>0.2178</v>
       </c>
       <c r="D54" t="n">
-        <v>0.2552</v>
+        <v>0.2596</v>
       </c>
       <c r="E54" t="n">
-        <v>0.2959</v>
+        <v>0.3027</v>
       </c>
       <c r="F54" t="n">
-        <v>0.3315</v>
+        <v>0.3407</v>
       </c>
       <c r="G54" t="n">
-        <v>0.3744</v>
+        <v>0.386</v>
       </c>
       <c r="H54" t="n">
-        <v>0.4133</v>
+        <v>0.4273</v>
       </c>
       <c r="I54" t="n">
-        <v>0.4515</v>
+        <v>0.4678</v>
       </c>
       <c r="J54" t="n">
-        <v>0.4907</v>
+        <v>0.5093</v>
       </c>
       <c r="K54" t="n">
-        <v>0.5284</v>
+        <v>0.5493</v>
       </c>
       <c r="L54" t="n">
-        <v>0.5668</v>
+        <v>0.5901</v>
       </c>
       <c r="M54" t="n">
-        <v>0.6062</v>
+        <v>0.6318</v>
       </c>
       <c r="N54" t="n">
-        <v>0.6425999999999999</v>
+        <v>0.6706</v>
       </c>
       <c r="O54" t="n">
-        <v>0.6772</v>
+        <v>0.7073</v>
       </c>
       <c r="P54" t="n">
-        <v>0.719</v>
+        <v>0.7516</v>
       </c>
       <c r="Q54" t="n">
-        <v>0.754</v>
+        <v>0.7887999999999999</v>
       </c>
       <c r="R54" t="n">
-        <v>0.7927</v>
+        <v>0.83</v>
       </c>
       <c r="S54" t="n">
-        <v>0.8305</v>
+        <v>0.8701</v>
       </c>
       <c r="T54" t="n">
-        <v>0.8649</v>
+        <v>0.9068000000000001</v>
       </c>
       <c r="U54" t="n">
-        <v>0.902</v>
+        <v>0.9462</v>
       </c>
       <c r="V54" t="n">
-        <v>0.9433</v>
+        <v>0.9899</v>
       </c>
       <c r="W54" t="n">
-        <v>0.9745</v>
+        <v>1.0231</v>
       </c>
       <c r="X54" t="n">
-        <v>1.0172</v>
+        <v>1.0685</v>
       </c>
       <c r="Y54" t="n">
-        <v>1.0478</v>
+        <v>1.1012</v>
       </c>
       <c r="Z54" t="n">
-        <v>1.0884</v>
+        <v>1.1443</v>
       </c>
       <c r="AA54" t="n">
-        <v>1.1154</v>
+        <v>1.1733</v>
       </c>
       <c r="AB54" t="n">
-        <v>1.1563</v>
+        <v>1.2166</v>
       </c>
       <c r="AC54" t="n">
-        <v>1.1966</v>
+        <v>1.2596</v>
       </c>
       <c r="AD54" t="n">
-        <v>1.229</v>
+        <v>1.2941</v>
       </c>
       <c r="AE54" t="n">
-        <v>1.266</v>
+        <v>1.3334</v>
       </c>
       <c r="AF54" t="n">
-        <v>1.2992</v>
+        <v>1.3688</v>
       </c>
       <c r="AG54" t="n">
-        <v>1.3305</v>
+        <v>1.4021</v>
       </c>
       <c r="AH54" t="n">
-        <v>1.3758</v>
+        <v>1.4504</v>
       </c>
       <c r="AI54" t="n">
-        <v>1.3996</v>
+        <v>1.4759</v>
       </c>
       <c r="AJ54" t="n">
-        <v>1.4376</v>
+        <v>1.5164</v>
       </c>
       <c r="AK54" t="n">
-        <v>1.4745</v>
+        <v>1.5557</v>
       </c>
       <c r="AL54" t="n">
-        <v>1.5076</v>
+        <v>1.5912</v>
       </c>
     </row>
     <row r="55">
@@ -3176,112 +3176,112 @@
         <v>0.158</v>
       </c>
       <c r="C55" t="n">
-        <v>0.1861</v>
+        <v>0.1898</v>
       </c>
       <c r="D55" t="n">
-        <v>0.2261</v>
+        <v>0.234</v>
       </c>
       <c r="E55" t="n">
-        <v>0.2605</v>
+        <v>0.2726</v>
       </c>
       <c r="F55" t="n">
-        <v>0.3003</v>
+        <v>0.3168</v>
       </c>
       <c r="G55" t="n">
-        <v>0.3325</v>
+        <v>0.3529</v>
       </c>
       <c r="H55" t="n">
-        <v>0.3696</v>
+        <v>0.3944</v>
       </c>
       <c r="I55" t="n">
-        <v>0.4059</v>
+        <v>0.4346</v>
       </c>
       <c r="J55" t="n">
-        <v>0.4419</v>
+        <v>0.4749</v>
       </c>
       <c r="K55" t="n">
-        <v>0.474</v>
+        <v>0.5111</v>
       </c>
       <c r="L55" t="n">
-        <v>0.5125</v>
+        <v>0.5538999999999999</v>
       </c>
       <c r="M55" t="n">
-        <v>0.544</v>
+        <v>0.5894</v>
       </c>
       <c r="N55" t="n">
-        <v>0.5782</v>
+        <v>0.628</v>
       </c>
       <c r="O55" t="n">
-        <v>0.6157</v>
+        <v>0.6697</v>
       </c>
       <c r="P55" t="n">
-        <v>0.65</v>
+        <v>0.7083</v>
       </c>
       <c r="Q55" t="n">
-        <v>0.6823</v>
+        <v>0.7447</v>
       </c>
       <c r="R55" t="n">
-        <v>0.7173</v>
+        <v>0.7839</v>
       </c>
       <c r="S55" t="n">
-        <v>0.7514</v>
+        <v>0.8226</v>
       </c>
       <c r="T55" t="n">
-        <v>0.7822</v>
+        <v>0.8571</v>
       </c>
       <c r="U55" t="n">
-        <v>0.8183</v>
+        <v>0.8976</v>
       </c>
       <c r="V55" t="n">
-        <v>0.8539</v>
+        <v>0.9379</v>
       </c>
       <c r="W55" t="n">
-        <v>0.8808</v>
+        <v>0.9683</v>
       </c>
       <c r="X55" t="n">
-        <v>0.9224</v>
+        <v>1.0152</v>
       </c>
       <c r="Y55" t="n">
-        <v>0.9520999999999999</v>
+        <v>1.0489</v>
       </c>
       <c r="Z55" t="n">
-        <v>0.9782999999999999</v>
+        <v>1.0787</v>
       </c>
       <c r="AA55" t="n">
-        <v>1.0092</v>
+        <v>1.1138</v>
       </c>
       <c r="AB55" t="n">
-        <v>1.0483</v>
+        <v>1.1579</v>
       </c>
       <c r="AC55" t="n">
-        <v>1.0777</v>
+        <v>1.1915</v>
       </c>
       <c r="AD55" t="n">
-        <v>1.1053</v>
+        <v>1.2226</v>
       </c>
       <c r="AE55" t="n">
-        <v>1.1414</v>
+        <v>1.264</v>
       </c>
       <c r="AF55" t="n">
-        <v>1.1626</v>
+        <v>1.288</v>
       </c>
       <c r="AG55" t="n">
-        <v>1.1976</v>
+        <v>1.328</v>
       </c>
       <c r="AH55" t="n">
-        <v>1.2314</v>
+        <v>1.3663</v>
       </c>
       <c r="AI55" t="n">
-        <v>1.2627</v>
+        <v>1.4021</v>
       </c>
       <c r="AJ55" t="n">
-        <v>1.2902</v>
+        <v>1.4333</v>
       </c>
       <c r="AK55" t="n">
-        <v>1.3177</v>
+        <v>1.4651</v>
       </c>
       <c r="AL55" t="n">
-        <v>1.3483</v>
+        <v>1.4996</v>
       </c>
     </row>
     <row r="56">
@@ -3294,112 +3294,112 @@
         <v>0.1566</v>
       </c>
       <c r="C56" t="n">
-        <v>0.1869</v>
+        <v>0.1928</v>
       </c>
       <c r="D56" t="n">
-        <v>0.2169</v>
+        <v>0.2294</v>
       </c>
       <c r="E56" t="n">
-        <v>0.2513</v>
+        <v>0.2705</v>
       </c>
       <c r="F56" t="n">
-        <v>0.283</v>
+        <v>0.3086</v>
       </c>
       <c r="G56" t="n">
-        <v>0.3144</v>
+        <v>0.3468</v>
       </c>
       <c r="H56" t="n">
-        <v>0.3442</v>
+        <v>0.3833</v>
       </c>
       <c r="I56" t="n">
-        <v>0.3736</v>
+        <v>0.419</v>
       </c>
       <c r="J56" t="n">
-        <v>0.405</v>
+        <v>0.457</v>
       </c>
       <c r="K56" t="n">
-        <v>0.4369</v>
+        <v>0.4957</v>
       </c>
       <c r="L56" t="n">
-        <v>0.4623</v>
+        <v>0.527</v>
       </c>
       <c r="M56" t="n">
-        <v>0.4931</v>
+        <v>0.5645</v>
       </c>
       <c r="N56" t="n">
-        <v>0.5228</v>
+        <v>0.6007</v>
       </c>
       <c r="O56" t="n">
-        <v>0.5508999999999999</v>
+        <v>0.6347</v>
       </c>
       <c r="P56" t="n">
-        <v>0.5802</v>
+        <v>0.6705</v>
       </c>
       <c r="Q56" t="n">
-        <v>0.602</v>
+        <v>0.6977</v>
       </c>
       <c r="R56" t="n">
-        <v>0.6364</v>
+        <v>0.7392</v>
       </c>
       <c r="S56" t="n">
-        <v>0.6587</v>
+        <v>0.7665999999999999</v>
       </c>
       <c r="T56" t="n">
-        <v>0.6865</v>
+        <v>0.8007</v>
       </c>
       <c r="U56" t="n">
-        <v>0.7113</v>
+        <v>0.8316</v>
       </c>
       <c r="V56" t="n">
-        <v>0.7362</v>
+        <v>0.8616</v>
       </c>
       <c r="W56" t="n">
-        <v>0.7579</v>
+        <v>0.8882</v>
       </c>
       <c r="X56" t="n">
-        <v>0.7868000000000001</v>
+        <v>0.9235</v>
       </c>
       <c r="Y56" t="n">
-        <v>0.8173</v>
+        <v>0.9603</v>
       </c>
       <c r="Z56" t="n">
-        <v>0.836</v>
+        <v>0.9833</v>
       </c>
       <c r="AA56" t="n">
-        <v>0.8594000000000001</v>
+        <v>1.0112</v>
       </c>
       <c r="AB56" t="n">
-        <v>0.8825</v>
+        <v>1.0395</v>
       </c>
       <c r="AC56" t="n">
-        <v>0.9043</v>
+        <v>1.0648</v>
       </c>
       <c r="AD56" t="n">
-        <v>0.926</v>
+        <v>1.0912</v>
       </c>
       <c r="AE56" t="n">
-        <v>0.9473</v>
+        <v>1.1164</v>
       </c>
       <c r="AF56" t="n">
-        <v>0.9721</v>
+        <v>1.1463</v>
       </c>
       <c r="AG56" t="n">
-        <v>0.9886</v>
+        <v>1.1657</v>
       </c>
       <c r="AH56" t="n">
-        <v>1.0102</v>
+        <v>1.1906</v>
       </c>
       <c r="AI56" t="n">
-        <v>1.029</v>
+        <v>1.2119</v>
       </c>
       <c r="AJ56" t="n">
-        <v>1.052</v>
+        <v>1.2381</v>
       </c>
       <c r="AK56" t="n">
-        <v>1.07</v>
+        <v>1.2588</v>
       </c>
       <c r="AL56" t="n">
-        <v>1.0942</v>
+        <v>1.2858</v>
       </c>
     </row>
     <row r="57">
@@ -3412,112 +3412,112 @@
         <v>0.1821</v>
       </c>
       <c r="C57" t="n">
-        <v>0.2005</v>
+        <v>0.2074</v>
       </c>
       <c r="D57" t="n">
-        <v>0.2238</v>
+        <v>0.2383</v>
       </c>
       <c r="E57" t="n">
-        <v>0.2462</v>
+        <v>0.2682</v>
       </c>
       <c r="F57" t="n">
-        <v>0.2689</v>
+        <v>0.2985</v>
       </c>
       <c r="G57" t="n">
-        <v>0.2903</v>
+        <v>0.3269</v>
       </c>
       <c r="H57" t="n">
-        <v>0.3099</v>
+        <v>0.3536</v>
       </c>
       <c r="I57" t="n">
-        <v>0.3297</v>
+        <v>0.3801</v>
       </c>
       <c r="J57" t="n">
-        <v>0.3506</v>
+        <v>0.4075</v>
       </c>
       <c r="K57" t="n">
-        <v>0.3694</v>
+        <v>0.4333</v>
       </c>
       <c r="L57" t="n">
-        <v>0.3906</v>
+        <v>0.4605</v>
       </c>
       <c r="M57" t="n">
-        <v>0.4099</v>
+        <v>0.4858</v>
       </c>
       <c r="N57" t="n">
-        <v>0.4263</v>
+        <v>0.5078</v>
       </c>
       <c r="O57" t="n">
-        <v>0.446</v>
+        <v>0.5328000000000001</v>
       </c>
       <c r="P57" t="n">
-        <v>0.4626</v>
+        <v>0.5546</v>
       </c>
       <c r="Q57" t="n">
-        <v>0.4806</v>
+        <v>0.5769</v>
       </c>
       <c r="R57" t="n">
-        <v>0.4979</v>
+        <v>0.5985</v>
       </c>
       <c r="S57" t="n">
-        <v>0.51</v>
+        <v>0.6145</v>
       </c>
       <c r="T57" t="n">
-        <v>0.5292</v>
+        <v>0.6379</v>
       </c>
       <c r="U57" t="n">
-        <v>0.5427999999999999</v>
+        <v>0.6546</v>
       </c>
       <c r="V57" t="n">
-        <v>0.5595</v>
+        <v>0.6746</v>
       </c>
       <c r="W57" t="n">
-        <v>0.5737</v>
+        <v>0.6915</v>
       </c>
       <c r="X57" t="n">
-        <v>0.5838</v>
+        <v>0.7028</v>
       </c>
       <c r="Y57" t="n">
-        <v>0.6</v>
+        <v>0.7207</v>
       </c>
       <c r="Z57" t="n">
-        <v>0.6135</v>
+        <v>0.7358</v>
       </c>
       <c r="AA57" t="n">
-        <v>0.622</v>
+        <v>0.7442</v>
       </c>
       <c r="AB57" t="n">
-        <v>0.6346000000000001</v>
+        <v>0.7577</v>
       </c>
       <c r="AC57" t="n">
-        <v>0.6465</v>
+        <v>0.7698</v>
       </c>
       <c r="AD57" t="n">
-        <v>0.6588000000000001</v>
+        <v>0.7819</v>
       </c>
       <c r="AE57" t="n">
-        <v>0.6741</v>
+        <v>0.7972</v>
       </c>
       <c r="AF57" t="n">
-        <v>0.6796</v>
+        <v>0.8008</v>
       </c>
       <c r="AG57" t="n">
-        <v>0.6924</v>
+        <v>0.8127</v>
       </c>
       <c r="AH57" t="n">
-        <v>0.6976</v>
+        <v>0.8156</v>
       </c>
       <c r="AI57" t="n">
-        <v>0.7136</v>
+        <v>0.8303</v>
       </c>
       <c r="AJ57" t="n">
-        <v>0.7194</v>
+        <v>0.8338</v>
       </c>
       <c r="AK57" t="n">
-        <v>0.7275</v>
+        <v>0.8397</v>
       </c>
       <c r="AL57" t="n">
-        <v>0.7377</v>
+        <v>0.8469</v>
       </c>
     </row>
     <row r="58">
@@ -3530,112 +3530,112 @@
         <v>0.1874</v>
       </c>
       <c r="C58" t="n">
-        <v>0.2024</v>
+        <v>0.2089</v>
       </c>
       <c r="D58" t="n">
-        <v>0.2164</v>
+        <v>0.2298</v>
       </c>
       <c r="E58" t="n">
-        <v>0.23</v>
+        <v>0.2502</v>
       </c>
       <c r="F58" t="n">
-        <v>0.2461</v>
+        <v>0.2726</v>
       </c>
       <c r="G58" t="n">
-        <v>0.2565</v>
+        <v>0.2891</v>
       </c>
       <c r="H58" t="n">
-        <v>0.27</v>
+        <v>0.3078</v>
       </c>
       <c r="I58" t="n">
-        <v>0.2805</v>
+        <v>0.3237</v>
       </c>
       <c r="J58" t="n">
-        <v>0.2923</v>
+        <v>0.34</v>
       </c>
       <c r="K58" t="n">
-        <v>0.3044</v>
+        <v>0.3565</v>
       </c>
       <c r="L58" t="n">
-        <v>0.3147</v>
+        <v>0.3707</v>
       </c>
       <c r="M58" t="n">
-        <v>0.3247</v>
+        <v>0.3841</v>
       </c>
       <c r="N58" t="n">
-        <v>0.3372</v>
+        <v>0.3995</v>
       </c>
       <c r="O58" t="n">
-        <v>0.3458</v>
+        <v>0.4106</v>
       </c>
       <c r="P58" t="n">
-        <v>0.3542</v>
+        <v>0.4211</v>
       </c>
       <c r="Q58" t="n">
-        <v>0.366</v>
+        <v>0.4351</v>
       </c>
       <c r="R58" t="n">
-        <v>0.3726</v>
+        <v>0.4424</v>
       </c>
       <c r="S58" t="n">
-        <v>0.3812</v>
+        <v>0.4524</v>
       </c>
       <c r="T58" t="n">
-        <v>0.3896</v>
+        <v>0.4616</v>
       </c>
       <c r="U58" t="n">
-        <v>0.3984</v>
+        <v>0.4704</v>
       </c>
       <c r="V58" t="n">
-        <v>0.4048</v>
+        <v>0.4767</v>
       </c>
       <c r="W58" t="n">
-        <v>0.413</v>
+        <v>0.4847</v>
       </c>
       <c r="X58" t="n">
-        <v>0.4171</v>
+        <v>0.4878</v>
       </c>
       <c r="Y58" t="n">
-        <v>0.4264</v>
+        <v>0.4964</v>
       </c>
       <c r="Z58" t="n">
-        <v>0.4334</v>
+        <v>0.5024999999999999</v>
       </c>
       <c r="AA58" t="n">
-        <v>0.4377</v>
+        <v>0.5054</v>
       </c>
       <c r="AB58" t="n">
-        <v>0.4446</v>
+        <v>0.5112</v>
       </c>
       <c r="AC58" t="n">
-        <v>0.4475</v>
+        <v>0.5124</v>
       </c>
       <c r="AD58" t="n">
-        <v>0.4538</v>
+        <v>0.5172</v>
       </c>
       <c r="AE58" t="n">
-        <v>0.4595</v>
+        <v>0.5212</v>
       </c>
       <c r="AF58" t="n">
-        <v>0.4626</v>
+        <v>0.5226</v>
       </c>
       <c r="AG58" t="n">
-        <v>0.4705</v>
+        <v>0.5286</v>
       </c>
       <c r="AH58" t="n">
-        <v>0.4739</v>
+        <v>0.5299</v>
       </c>
       <c r="AI58" t="n">
-        <v>0.4778</v>
+        <v>0.5317</v>
       </c>
       <c r="AJ58" t="n">
-        <v>0.4825</v>
+        <v>0.5347</v>
       </c>
       <c r="AK58" t="n">
-        <v>0.4846</v>
+        <v>0.5344</v>
       </c>
       <c r="AL58" t="n">
-        <v>0.4893</v>
+        <v>0.5375</v>
       </c>
     </row>
     <row r="59">
@@ -3648,112 +3648,112 @@
         <v>0.1631</v>
       </c>
       <c r="C59" t="n">
-        <v>0.1634</v>
+        <v>0.1644</v>
       </c>
       <c r="D59" t="n">
-        <v>0.1671</v>
+        <v>0.1705</v>
       </c>
       <c r="E59" t="n">
-        <v>0.1731</v>
+        <v>0.1799</v>
       </c>
       <c r="F59" t="n">
-        <v>0.18</v>
+        <v>0.1906</v>
       </c>
       <c r="G59" t="n">
-        <v>0.1854</v>
+        <v>0.1999</v>
       </c>
       <c r="H59" t="n">
-        <v>0.1923</v>
+        <v>0.2106</v>
       </c>
       <c r="I59" t="n">
-        <v>0.1986</v>
+        <v>0.2206</v>
       </c>
       <c r="J59" t="n">
-        <v>0.2057</v>
+        <v>0.2311</v>
       </c>
       <c r="K59" t="n">
-        <v>0.2135</v>
+        <v>0.2418</v>
       </c>
       <c r="L59" t="n">
-        <v>0.2184</v>
+        <v>0.2493</v>
       </c>
       <c r="M59" t="n">
-        <v>0.2266</v>
+        <v>0.2599</v>
       </c>
       <c r="N59" t="n">
-        <v>0.231</v>
+        <v>0.266</v>
       </c>
       <c r="O59" t="n">
-        <v>0.2396</v>
+        <v>0.2764</v>
       </c>
       <c r="P59" t="n">
-        <v>0.2452</v>
+        <v>0.2829</v>
       </c>
       <c r="Q59" t="n">
-        <v>0.248</v>
+        <v>0.2867</v>
       </c>
       <c r="R59" t="n">
-        <v>0.255</v>
+        <v>0.2944</v>
       </c>
       <c r="S59" t="n">
-        <v>0.2587</v>
+        <v>0.2984</v>
       </c>
       <c r="T59" t="n">
-        <v>0.2647</v>
+        <v>0.3044</v>
       </c>
       <c r="U59" t="n">
-        <v>0.2683</v>
+        <v>0.3077</v>
       </c>
       <c r="V59" t="n">
-        <v>0.2723</v>
+        <v>0.3111</v>
       </c>
       <c r="W59" t="n">
-        <v>0.2753</v>
+        <v>0.3139</v>
       </c>
       <c r="X59" t="n">
-        <v>0.2769</v>
+        <v>0.3147</v>
       </c>
       <c r="Y59" t="n">
-        <v>0.2838</v>
+        <v>0.3208</v>
       </c>
       <c r="Z59" t="n">
-        <v>0.2866</v>
+        <v>0.3227</v>
       </c>
       <c r="AA59" t="n">
-        <v>0.2883</v>
+        <v>0.3232</v>
       </c>
       <c r="AB59" t="n">
-        <v>0.2945</v>
+        <v>0.3287</v>
       </c>
       <c r="AC59" t="n">
-        <v>0.296</v>
+        <v>0.3291</v>
       </c>
       <c r="AD59" t="n">
-        <v>0.2988</v>
+        <v>0.3307</v>
       </c>
       <c r="AE59" t="n">
-        <v>0.3003</v>
+        <v>0.3312</v>
       </c>
       <c r="AF59" t="n">
-        <v>0.303</v>
+        <v>0.3326</v>
       </c>
       <c r="AG59" t="n">
-        <v>0.3061</v>
+        <v>0.3348</v>
       </c>
       <c r="AH59" t="n">
-        <v>0.3089</v>
+        <v>0.3361</v>
       </c>
       <c r="AI59" t="n">
-        <v>0.3107</v>
+        <v>0.3369</v>
       </c>
       <c r="AJ59" t="n">
-        <v>0.311</v>
+        <v>0.336</v>
       </c>
       <c r="AK59" t="n">
-        <v>0.314</v>
+        <v>0.3379</v>
       </c>
       <c r="AL59" t="n">
-        <v>0.3161</v>
+        <v>0.3388</v>
       </c>
     </row>
     <row r="60">
@@ -3890,106 +3890,106 @@
         <v>0.1854</v>
       </c>
       <c r="E61" t="n">
-        <v>0.2073</v>
+        <v>0.2074</v>
       </c>
       <c r="F61" t="n">
-        <v>0.2324</v>
+        <v>0.2325</v>
       </c>
       <c r="G61" t="n">
-        <v>0.2604</v>
+        <v>0.2606</v>
       </c>
       <c r="H61" t="n">
-        <v>0.293</v>
+        <v>0.2932</v>
       </c>
       <c r="I61" t="n">
-        <v>0.3226</v>
+        <v>0.3229</v>
       </c>
       <c r="J61" t="n">
-        <v>0.3595</v>
+        <v>0.3599</v>
       </c>
       <c r="K61" t="n">
-        <v>0.3906</v>
+        <v>0.3909</v>
       </c>
       <c r="L61" t="n">
-        <v>0.4264</v>
+        <v>0.4268</v>
       </c>
       <c r="M61" t="n">
-        <v>0.4625</v>
+        <v>0.463</v>
       </c>
       <c r="N61" t="n">
-        <v>0.4974</v>
+        <v>0.4979</v>
       </c>
       <c r="O61" t="n">
-        <v>0.5309</v>
+        <v>0.5315</v>
       </c>
       <c r="P61" t="n">
-        <v>0.5647</v>
+        <v>0.5653</v>
       </c>
       <c r="Q61" t="n">
-        <v>0.5972</v>
+        <v>0.5979</v>
       </c>
       <c r="R61" t="n">
-        <v>0.6337</v>
+        <v>0.6345</v>
       </c>
       <c r="S61" t="n">
-        <v>0.6689000000000001</v>
+        <v>0.6696</v>
       </c>
       <c r="T61" t="n">
-        <v>0.7038</v>
+        <v>0.7046</v>
       </c>
       <c r="U61" t="n">
-        <v>0.7423</v>
+        <v>0.7432</v>
       </c>
       <c r="V61" t="n">
-        <v>0.7695</v>
+        <v>0.7705</v>
       </c>
       <c r="W61" t="n">
-        <v>0.8052</v>
+        <v>0.8062</v>
       </c>
       <c r="X61" t="n">
-        <v>0.8406</v>
+        <v>0.8416</v>
       </c>
       <c r="Y61" t="n">
-        <v>0.8732</v>
+        <v>0.8743</v>
       </c>
       <c r="Z61" t="n">
-        <v>0.908</v>
+        <v>0.9092</v>
       </c>
       <c r="AA61" t="n">
-        <v>0.9432</v>
+        <v>0.9444</v>
       </c>
       <c r="AB61" t="n">
-        <v>0.977</v>
+        <v>0.9782999999999999</v>
       </c>
       <c r="AC61" t="n">
-        <v>1.0101</v>
+        <v>1.0114</v>
       </c>
       <c r="AD61" t="n">
-        <v>1.0393</v>
+        <v>1.0406</v>
       </c>
       <c r="AE61" t="n">
-        <v>1.0784</v>
+        <v>1.0798</v>
       </c>
       <c r="AF61" t="n">
-        <v>1.113</v>
+        <v>1.1145</v>
       </c>
       <c r="AG61" t="n">
-        <v>1.1468</v>
+        <v>1.1483</v>
       </c>
       <c r="AH61" t="n">
-        <v>1.174</v>
+        <v>1.1755</v>
       </c>
       <c r="AI61" t="n">
-        <v>1.2045</v>
+        <v>1.2061</v>
       </c>
       <c r="AJ61" t="n">
-        <v>1.2334</v>
+        <v>1.235</v>
       </c>
       <c r="AK61" t="n">
-        <v>1.2778</v>
+        <v>1.2795</v>
       </c>
       <c r="AL61" t="n">
-        <v>1.3083</v>
+        <v>1.3101</v>
       </c>
     </row>
     <row r="62">
@@ -4002,112 +4002,112 @@
         <v>0.1722</v>
       </c>
       <c r="C62" t="n">
-        <v>0.2111</v>
+        <v>0.2112</v>
       </c>
       <c r="D62" t="n">
-        <v>0.2519</v>
+        <v>0.2522</v>
       </c>
       <c r="E62" t="n">
-        <v>0.2962</v>
+        <v>0.2966</v>
       </c>
       <c r="F62" t="n">
-        <v>0.3377</v>
+        <v>0.3383</v>
       </c>
       <c r="G62" t="n">
-        <v>0.3801</v>
+        <v>0.3808</v>
       </c>
       <c r="H62" t="n">
-        <v>0.4237</v>
+        <v>0.4245</v>
       </c>
       <c r="I62" t="n">
-        <v>0.4633</v>
+        <v>0.4644</v>
       </c>
       <c r="J62" t="n">
-        <v>0.5004</v>
+        <v>0.5014999999999999</v>
       </c>
       <c r="K62" t="n">
-        <v>0.5424</v>
+        <v>0.5437</v>
       </c>
       <c r="L62" t="n">
-        <v>0.5862000000000001</v>
+        <v>0.5877</v>
       </c>
       <c r="M62" t="n">
-        <v>0.6337</v>
+        <v>0.6353</v>
       </c>
       <c r="N62" t="n">
-        <v>0.6708</v>
+        <v>0.6725</v>
       </c>
       <c r="O62" t="n">
-        <v>0.7125</v>
+        <v>0.7143</v>
       </c>
       <c r="P62" t="n">
-        <v>0.7527</v>
+        <v>0.7547</v>
       </c>
       <c r="Q62" t="n">
-        <v>0.7923</v>
+        <v>0.7945</v>
       </c>
       <c r="R62" t="n">
-        <v>0.8364</v>
+        <v>0.8387</v>
       </c>
       <c r="S62" t="n">
-        <v>0.876</v>
+        <v>0.8784999999999999</v>
       </c>
       <c r="T62" t="n">
-        <v>0.9156</v>
+        <v>0.9182</v>
       </c>
       <c r="U62" t="n">
-        <v>0.9575</v>
+        <v>0.9602000000000001</v>
       </c>
       <c r="V62" t="n">
-        <v>0.9994</v>
+        <v>1.0023</v>
       </c>
       <c r="W62" t="n">
-        <v>1.0374</v>
+        <v>1.0403</v>
       </c>
       <c r="X62" t="n">
-        <v>1.0767</v>
+        <v>1.0798</v>
       </c>
       <c r="Y62" t="n">
-        <v>1.1139</v>
+        <v>1.1171</v>
       </c>
       <c r="Z62" t="n">
-        <v>1.1477</v>
+        <v>1.151</v>
       </c>
       <c r="AA62" t="n">
-        <v>1.1876</v>
+        <v>1.1911</v>
       </c>
       <c r="AB62" t="n">
-        <v>1.2271</v>
+        <v>1.2307</v>
       </c>
       <c r="AC62" t="n">
-        <v>1.271</v>
+        <v>1.2747</v>
       </c>
       <c r="AD62" t="n">
-        <v>1.3108</v>
+        <v>1.3147</v>
       </c>
       <c r="AE62" t="n">
-        <v>1.351</v>
+        <v>1.355</v>
       </c>
       <c r="AF62" t="n">
-        <v>1.3868</v>
+        <v>1.391</v>
       </c>
       <c r="AG62" t="n">
-        <v>1.4274</v>
+        <v>1.4317</v>
       </c>
       <c r="AH62" t="n">
-        <v>1.4627</v>
+        <v>1.467</v>
       </c>
       <c r="AI62" t="n">
-        <v>1.4957</v>
+        <v>1.5002</v>
       </c>
       <c r="AJ62" t="n">
-        <v>1.5435</v>
+        <v>1.5482</v>
       </c>
       <c r="AK62" t="n">
-        <v>1.5818</v>
+        <v>1.5865</v>
       </c>
       <c r="AL62" t="n">
-        <v>1.6214</v>
+        <v>1.6262</v>
       </c>
     </row>
     <row r="63">
@@ -4120,112 +4120,112 @@
         <v>0.1636</v>
       </c>
       <c r="C63" t="n">
-        <v>0.2046</v>
+        <v>0.2048</v>
       </c>
       <c r="D63" t="n">
-        <v>0.2441</v>
+        <v>0.2446</v>
       </c>
       <c r="E63" t="n">
-        <v>0.2883</v>
+        <v>0.2892</v>
       </c>
       <c r="F63" t="n">
-        <v>0.3258</v>
+        <v>0.327</v>
       </c>
       <c r="G63" t="n">
-        <v>0.3665</v>
+        <v>0.368</v>
       </c>
       <c r="H63" t="n">
-        <v>0.4084</v>
+        <v>0.4102</v>
       </c>
       <c r="I63" t="n">
-        <v>0.4479</v>
+        <v>0.45</v>
       </c>
       <c r="J63" t="n">
-        <v>0.4904</v>
+        <v>0.4927</v>
       </c>
       <c r="K63" t="n">
-        <v>0.5271</v>
+        <v>0.5298</v>
       </c>
       <c r="L63" t="n">
-        <v>0.5694</v>
+        <v>0.5724</v>
       </c>
       <c r="M63" t="n">
-        <v>0.6127</v>
+        <v>0.6159</v>
       </c>
       <c r="N63" t="n">
-        <v>0.6482</v>
+        <v>0.6518</v>
       </c>
       <c r="O63" t="n">
-        <v>0.6909</v>
+        <v>0.6948</v>
       </c>
       <c r="P63" t="n">
-        <v>0.7295</v>
+        <v>0.7337</v>
       </c>
       <c r="Q63" t="n">
-        <v>0.7607</v>
+        <v>0.7651</v>
       </c>
       <c r="R63" t="n">
-        <v>0.804</v>
+        <v>0.8086</v>
       </c>
       <c r="S63" t="n">
-        <v>0.8476</v>
+        <v>0.8526</v>
       </c>
       <c r="T63" t="n">
-        <v>0.8806</v>
+        <v>0.8858</v>
       </c>
       <c r="U63" t="n">
-        <v>0.9243</v>
+        <v>0.9298</v>
       </c>
       <c r="V63" t="n">
-        <v>0.9639</v>
+        <v>0.9697</v>
       </c>
       <c r="W63" t="n">
-        <v>0.9983</v>
+        <v>1.0044</v>
       </c>
       <c r="X63" t="n">
-        <v>1.0368</v>
+        <v>1.0431</v>
       </c>
       <c r="Y63" t="n">
-        <v>1.0784</v>
+        <v>1.085</v>
       </c>
       <c r="Z63" t="n">
-        <v>1.1178</v>
+        <v>1.1246</v>
       </c>
       <c r="AA63" t="n">
-        <v>1.1501</v>
+        <v>1.1573</v>
       </c>
       <c r="AB63" t="n">
-        <v>1.1941</v>
+        <v>1.2015</v>
       </c>
       <c r="AC63" t="n">
-        <v>1.2298</v>
+        <v>1.2375</v>
       </c>
       <c r="AD63" t="n">
-        <v>1.2772</v>
+        <v>1.2852</v>
       </c>
       <c r="AE63" t="n">
-        <v>1.3091</v>
+        <v>1.3173</v>
       </c>
       <c r="AF63" t="n">
-        <v>1.3454</v>
+        <v>1.3539</v>
       </c>
       <c r="AG63" t="n">
-        <v>1.3752</v>
+        <v>1.3839</v>
       </c>
       <c r="AH63" t="n">
-        <v>1.4198</v>
+        <v>1.4288</v>
       </c>
       <c r="AI63" t="n">
-        <v>1.4584</v>
+        <v>1.4676</v>
       </c>
       <c r="AJ63" t="n">
-        <v>1.4993</v>
+        <v>1.5088</v>
       </c>
       <c r="AK63" t="n">
-        <v>1.5275</v>
+        <v>1.5372</v>
       </c>
       <c r="AL63" t="n">
-        <v>1.5684</v>
+        <v>1.5784</v>
       </c>
     </row>
     <row r="64">
@@ -4238,112 +4238,112 @@
         <v>0.1713</v>
       </c>
       <c r="C64" t="n">
-        <v>0.2104</v>
+        <v>0.211</v>
       </c>
       <c r="D64" t="n">
-        <v>0.253</v>
+        <v>0.2542</v>
       </c>
       <c r="E64" t="n">
-        <v>0.2997</v>
+        <v>0.3017</v>
       </c>
       <c r="F64" t="n">
-        <v>0.3398</v>
+        <v>0.3423</v>
       </c>
       <c r="G64" t="n">
-        <v>0.3851</v>
+        <v>0.3883</v>
       </c>
       <c r="H64" t="n">
-        <v>0.4292</v>
+        <v>0.433</v>
       </c>
       <c r="I64" t="n">
-        <v>0.4693</v>
+        <v>0.4738</v>
       </c>
       <c r="J64" t="n">
-        <v>0.5141</v>
+        <v>0.5192</v>
       </c>
       <c r="K64" t="n">
-        <v>0.5543</v>
+        <v>0.5601</v>
       </c>
       <c r="L64" t="n">
-        <v>0.5965</v>
+        <v>0.6029</v>
       </c>
       <c r="M64" t="n">
-        <v>0.643</v>
+        <v>0.6501</v>
       </c>
       <c r="N64" t="n">
-        <v>0.6832</v>
+        <v>0.6909</v>
       </c>
       <c r="O64" t="n">
-        <v>0.723</v>
+        <v>0.7313</v>
       </c>
       <c r="P64" t="n">
-        <v>0.7661</v>
+        <v>0.775</v>
       </c>
       <c r="Q64" t="n">
-        <v>0.8062</v>
+        <v>0.8157</v>
       </c>
       <c r="R64" t="n">
-        <v>0.8466</v>
+        <v>0.8567</v>
       </c>
       <c r="S64" t="n">
-        <v>0.8933</v>
+        <v>0.9041</v>
       </c>
       <c r="T64" t="n">
-        <v>0.9321</v>
+        <v>0.9434</v>
       </c>
       <c r="U64" t="n">
-        <v>0.9717</v>
+        <v>0.9836</v>
       </c>
       <c r="V64" t="n">
-        <v>1.0133</v>
+        <v>1.0259</v>
       </c>
       <c r="W64" t="n">
-        <v>1.0551</v>
+        <v>1.0683</v>
       </c>
       <c r="X64" t="n">
-        <v>1.094</v>
+        <v>1.1078</v>
       </c>
       <c r="Y64" t="n">
-        <v>1.1392</v>
+        <v>1.1537</v>
       </c>
       <c r="Z64" t="n">
-        <v>1.176</v>
+        <v>1.191</v>
       </c>
       <c r="AA64" t="n">
-        <v>1.2178</v>
+        <v>1.2334</v>
       </c>
       <c r="AB64" t="n">
-        <v>1.2569</v>
+        <v>1.2731</v>
       </c>
       <c r="AC64" t="n">
-        <v>1.2975</v>
+        <v>1.3143</v>
       </c>
       <c r="AD64" t="n">
-        <v>1.3355</v>
+        <v>1.3528</v>
       </c>
       <c r="AE64" t="n">
-        <v>1.3708</v>
+        <v>1.3887</v>
       </c>
       <c r="AF64" t="n">
-        <v>1.4156</v>
+        <v>1.4341</v>
       </c>
       <c r="AG64" t="n">
-        <v>1.4581</v>
+        <v>1.4772</v>
       </c>
       <c r="AH64" t="n">
-        <v>1.4906</v>
+        <v>1.5102</v>
       </c>
       <c r="AI64" t="n">
-        <v>1.5404</v>
+        <v>1.5606</v>
       </c>
       <c r="AJ64" t="n">
-        <v>1.5697</v>
+        <v>1.5904</v>
       </c>
       <c r="AK64" t="n">
-        <v>1.6056</v>
+        <v>1.6269</v>
       </c>
       <c r="AL64" t="n">
-        <v>1.6461</v>
+        <v>1.668</v>
       </c>
     </row>
     <row r="65">
@@ -4356,112 +4356,112 @@
         <v>0.178</v>
       </c>
       <c r="C65" t="n">
-        <v>0.2166</v>
+        <v>0.2178</v>
       </c>
       <c r="D65" t="n">
-        <v>0.2598</v>
+        <v>0.2623</v>
       </c>
       <c r="E65" t="n">
-        <v>0.3039</v>
+        <v>0.3077</v>
       </c>
       <c r="F65" t="n">
-        <v>0.3491</v>
+        <v>0.3543</v>
       </c>
       <c r="G65" t="n">
-        <v>0.3914</v>
+        <v>0.3979</v>
       </c>
       <c r="H65" t="n">
-        <v>0.433</v>
+        <v>0.4407</v>
       </c>
       <c r="I65" t="n">
-        <v>0.4762</v>
+        <v>0.4853</v>
       </c>
       <c r="J65" t="n">
-        <v>0.5207000000000001</v>
+        <v>0.5312</v>
       </c>
       <c r="K65" t="n">
-        <v>0.5635</v>
+        <v>0.5753</v>
       </c>
       <c r="L65" t="n">
-        <v>0.6047</v>
+        <v>0.6177</v>
       </c>
       <c r="M65" t="n">
-        <v>0.6467000000000001</v>
+        <v>0.661</v>
       </c>
       <c r="N65" t="n">
-        <v>0.6887</v>
+        <v>0.7043</v>
       </c>
       <c r="O65" t="n">
-        <v>0.7302999999999999</v>
+        <v>0.7471</v>
       </c>
       <c r="P65" t="n">
-        <v>0.7753</v>
+        <v>0.7934</v>
       </c>
       <c r="Q65" t="n">
-        <v>0.8152</v>
+        <v>0.8346</v>
       </c>
       <c r="R65" t="n">
-        <v>0.8539</v>
+        <v>0.8745000000000001</v>
       </c>
       <c r="S65" t="n">
-        <v>0.8991</v>
+        <v>0.9211</v>
       </c>
       <c r="T65" t="n">
-        <v>0.9377</v>
+        <v>0.9608</v>
       </c>
       <c r="U65" t="n">
-        <v>0.9802</v>
+        <v>1.0046</v>
       </c>
       <c r="V65" t="n">
-        <v>1.0198</v>
+        <v>1.0454</v>
       </c>
       <c r="W65" t="n">
-        <v>1.0606</v>
+        <v>1.0874</v>
       </c>
       <c r="X65" t="n">
-        <v>1.1</v>
+        <v>1.1281</v>
       </c>
       <c r="Y65" t="n">
-        <v>1.1436</v>
+        <v>1.173</v>
       </c>
       <c r="Z65" t="n">
-        <v>1.1837</v>
+        <v>1.2144</v>
       </c>
       <c r="AA65" t="n">
-        <v>1.2211</v>
+        <v>1.2529</v>
       </c>
       <c r="AB65" t="n">
-        <v>1.2622</v>
+        <v>1.2952</v>
       </c>
       <c r="AC65" t="n">
-        <v>1.3021</v>
+        <v>1.3364</v>
       </c>
       <c r="AD65" t="n">
-        <v>1.3447</v>
+        <v>1.3803</v>
       </c>
       <c r="AE65" t="n">
-        <v>1.3874</v>
+        <v>1.4243</v>
       </c>
       <c r="AF65" t="n">
-        <v>1.4249</v>
+        <v>1.4629</v>
       </c>
       <c r="AG65" t="n">
-        <v>1.4583</v>
+        <v>1.4974</v>
       </c>
       <c r="AH65" t="n">
-        <v>1.5003</v>
+        <v>1.5407</v>
       </c>
       <c r="AI65" t="n">
-        <v>1.5414</v>
+        <v>1.5831</v>
       </c>
       <c r="AJ65" t="n">
-        <v>1.577</v>
+        <v>1.6198</v>
       </c>
       <c r="AK65" t="n">
-        <v>1.6182</v>
+        <v>1.6622</v>
       </c>
       <c r="AL65" t="n">
-        <v>1.6536</v>
+        <v>1.6987</v>
       </c>
     </row>
     <row r="66">
@@ -4474,112 +4474,112 @@
         <v>0.1745</v>
       </c>
       <c r="C66" t="n">
-        <v>0.2124</v>
+        <v>0.2146</v>
       </c>
       <c r="D66" t="n">
-        <v>0.2568</v>
+        <v>0.2616</v>
       </c>
       <c r="E66" t="n">
-        <v>0.2967</v>
+        <v>0.304</v>
       </c>
       <c r="F66" t="n">
-        <v>0.3405</v>
+        <v>0.3504</v>
       </c>
       <c r="G66" t="n">
-        <v>0.3807</v>
+        <v>0.393</v>
       </c>
       <c r="H66" t="n">
-        <v>0.4266</v>
+        <v>0.4416</v>
       </c>
       <c r="I66" t="n">
-        <v>0.469</v>
+        <v>0.4865</v>
       </c>
       <c r="J66" t="n">
-        <v>0.5081</v>
+        <v>0.5281</v>
       </c>
       <c r="K66" t="n">
-        <v>0.5488</v>
+        <v>0.5714</v>
       </c>
       <c r="L66" t="n">
-        <v>0.5927</v>
+        <v>0.6178</v>
       </c>
       <c r="M66" t="n">
-        <v>0.6356000000000001</v>
+        <v>0.6634</v>
       </c>
       <c r="N66" t="n">
-        <v>0.6757</v>
+        <v>0.7059</v>
       </c>
       <c r="O66" t="n">
-        <v>0.713</v>
+        <v>0.7456</v>
       </c>
       <c r="P66" t="n">
-        <v>0.7558</v>
+        <v>0.7911</v>
       </c>
       <c r="Q66" t="n">
-        <v>0.7943</v>
+        <v>0.832</v>
       </c>
       <c r="R66" t="n">
-        <v>0.8332000000000001</v>
+        <v>0.8733</v>
       </c>
       <c r="S66" t="n">
-        <v>0.8707</v>
+        <v>0.9132</v>
       </c>
       <c r="T66" t="n">
-        <v>0.9127999999999999</v>
+        <v>0.9579</v>
       </c>
       <c r="U66" t="n">
-        <v>0.9568</v>
+        <v>1.0047</v>
       </c>
       <c r="V66" t="n">
-        <v>0.996</v>
+        <v>1.0463</v>
       </c>
       <c r="W66" t="n">
-        <v>1.0392</v>
+        <v>1.0923</v>
       </c>
       <c r="X66" t="n">
-        <v>1.0711</v>
+        <v>1.1264</v>
       </c>
       <c r="Y66" t="n">
-        <v>1.11</v>
+        <v>1.1677</v>
       </c>
       <c r="Z66" t="n">
-        <v>1.1446</v>
+        <v>1.2045</v>
       </c>
       <c r="AA66" t="n">
-        <v>1.1847</v>
+        <v>1.2473</v>
       </c>
       <c r="AB66" t="n">
-        <v>1.2291</v>
+        <v>1.2946</v>
       </c>
       <c r="AC66" t="n">
-        <v>1.2652</v>
+        <v>1.3329</v>
       </c>
       <c r="AD66" t="n">
-        <v>1.3005</v>
+        <v>1.3706</v>
       </c>
       <c r="AE66" t="n">
-        <v>1.3366</v>
+        <v>1.4091</v>
       </c>
       <c r="AF66" t="n">
-        <v>1.3825</v>
+        <v>1.458</v>
       </c>
       <c r="AG66" t="n">
-        <v>1.4234</v>
+        <v>1.5017</v>
       </c>
       <c r="AH66" t="n">
-        <v>1.4512</v>
+        <v>1.5314</v>
       </c>
       <c r="AI66" t="n">
-        <v>1.4879</v>
+        <v>1.5706</v>
       </c>
       <c r="AJ66" t="n">
-        <v>1.5238</v>
+        <v>1.6089</v>
       </c>
       <c r="AK66" t="n">
-        <v>1.5585</v>
+        <v>1.646</v>
       </c>
       <c r="AL66" t="n">
-        <v>1.6015</v>
+        <v>1.6919</v>
       </c>
     </row>
     <row r="67">
@@ -4592,112 +4592,112 @@
         <v>0.1687</v>
       </c>
       <c r="C67" t="n">
-        <v>0.173</v>
+        <v>0.1735</v>
       </c>
       <c r="D67" t="n">
-        <v>0.1866</v>
+        <v>0.1885</v>
       </c>
       <c r="E67" t="n">
-        <v>0.2039</v>
+        <v>0.2078</v>
       </c>
       <c r="F67" t="n">
-        <v>0.2272</v>
+        <v>0.2335</v>
       </c>
       <c r="G67" t="n">
-        <v>0.2515</v>
+        <v>0.2606</v>
       </c>
       <c r="H67" t="n">
-        <v>0.2797</v>
+        <v>0.2919</v>
       </c>
       <c r="I67" t="n">
-        <v>0.3054</v>
+        <v>0.3208</v>
       </c>
       <c r="J67" t="n">
-        <v>0.3339</v>
+        <v>0.3527</v>
       </c>
       <c r="K67" t="n">
-        <v>0.3648</v>
+        <v>0.3871</v>
       </c>
       <c r="L67" t="n">
-        <v>0.3928</v>
+        <v>0.4186</v>
       </c>
       <c r="M67" t="n">
-        <v>0.428</v>
+        <v>0.4576</v>
       </c>
       <c r="N67" t="n">
-        <v>0.4572</v>
+        <v>0.4903</v>
       </c>
       <c r="O67" t="n">
-        <v>0.4897</v>
+        <v>0.5266999999999999</v>
       </c>
       <c r="P67" t="n">
-        <v>0.5167</v>
+        <v>0.5571</v>
       </c>
       <c r="Q67" t="n">
-        <v>0.5487</v>
+        <v>0.593</v>
       </c>
       <c r="R67" t="n">
-        <v>0.5797</v>
+        <v>0.6277</v>
       </c>
       <c r="S67" t="n">
-        <v>0.6118</v>
+        <v>0.6635</v>
       </c>
       <c r="T67" t="n">
-        <v>0.6461</v>
+        <v>0.7019</v>
       </c>
       <c r="U67" t="n">
-        <v>0.6716</v>
+        <v>0.7306</v>
       </c>
       <c r="V67" t="n">
-        <v>0.7022</v>
+        <v>0.7651</v>
       </c>
       <c r="W67" t="n">
-        <v>0.7316</v>
+        <v>0.7984</v>
       </c>
       <c r="X67" t="n">
-        <v>0.7647</v>
+        <v>0.8356</v>
       </c>
       <c r="Y67" t="n">
-        <v>0.794</v>
+        <v>0.8685</v>
       </c>
       <c r="Z67" t="n">
-        <v>0.8249</v>
+        <v>0.9034</v>
       </c>
       <c r="AA67" t="n">
-        <v>0.8514</v>
+        <v>0.9334</v>
       </c>
       <c r="AB67" t="n">
-        <v>0.8821</v>
+        <v>0.9679</v>
       </c>
       <c r="AC67" t="n">
-        <v>0.9091</v>
+        <v>0.9986</v>
       </c>
       <c r="AD67" t="n">
-        <v>0.9397</v>
+        <v>1.0332</v>
       </c>
       <c r="AE67" t="n">
-        <v>0.9756</v>
+        <v>1.0733</v>
       </c>
       <c r="AF67" t="n">
-        <v>1.0006</v>
+        <v>1.1019</v>
       </c>
       <c r="AG67" t="n">
-        <v>1.0259</v>
+        <v>1.1307</v>
       </c>
       <c r="AH67" t="n">
-        <v>1.0515</v>
+        <v>1.1597</v>
       </c>
       <c r="AI67" t="n">
-        <v>1.0862</v>
+        <v>1.199</v>
       </c>
       <c r="AJ67" t="n">
-        <v>1.1182</v>
+        <v>1.2353</v>
       </c>
       <c r="AK67" t="n">
-        <v>1.1354</v>
+        <v>1.2551</v>
       </c>
       <c r="AL67" t="n">
-        <v>1.1662</v>
+        <v>1.29</v>
       </c>
     </row>
     <row r="68">
@@ -4710,112 +4710,112 @@
         <v>0.1749</v>
       </c>
       <c r="C68" t="n">
-        <v>0.2015</v>
+        <v>0.2068</v>
       </c>
       <c r="D68" t="n">
-        <v>0.2305</v>
+        <v>0.2419</v>
       </c>
       <c r="E68" t="n">
-        <v>0.2592</v>
+        <v>0.2765</v>
       </c>
       <c r="F68" t="n">
-        <v>0.2876</v>
+        <v>0.3108</v>
       </c>
       <c r="G68" t="n">
-        <v>0.3156</v>
+        <v>0.3449</v>
       </c>
       <c r="H68" t="n">
-        <v>0.3438</v>
+        <v>0.3791</v>
       </c>
       <c r="I68" t="n">
-        <v>0.3722</v>
+        <v>0.4132</v>
       </c>
       <c r="J68" t="n">
-        <v>0.4007</v>
+        <v>0.4479</v>
       </c>
       <c r="K68" t="n">
-        <v>0.4267</v>
+        <v>0.4798</v>
       </c>
       <c r="L68" t="n">
-        <v>0.4521</v>
+        <v>0.5108</v>
       </c>
       <c r="M68" t="n">
-        <v>0.4822</v>
+        <v>0.547</v>
       </c>
       <c r="N68" t="n">
-        <v>0.5077</v>
+        <v>0.5783</v>
       </c>
       <c r="O68" t="n">
-        <v>0.5337</v>
+        <v>0.6101</v>
       </c>
       <c r="P68" t="n">
-        <v>0.5594</v>
+        <v>0.6415999999999999</v>
       </c>
       <c r="Q68" t="n">
-        <v>0.5835</v>
+        <v>0.6712</v>
       </c>
       <c r="R68" t="n">
-        <v>0.6106</v>
+        <v>0.7039</v>
       </c>
       <c r="S68" t="n">
-        <v>0.6354</v>
+        <v>0.7342</v>
       </c>
       <c r="T68" t="n">
-        <v>0.658</v>
+        <v>0.7619</v>
       </c>
       <c r="U68" t="n">
-        <v>0.6828</v>
+        <v>0.7925</v>
       </c>
       <c r="V68" t="n">
-        <v>0.7062</v>
+        <v>0.8206</v>
       </c>
       <c r="W68" t="n">
-        <v>0.7297</v>
+        <v>0.8495</v>
       </c>
       <c r="X68" t="n">
-        <v>0.7514</v>
+        <v>0.8761</v>
       </c>
       <c r="Y68" t="n">
-        <v>0.7739</v>
+        <v>0.9038</v>
       </c>
       <c r="Z68" t="n">
-        <v>0.7993</v>
+        <v>0.9340000000000001</v>
       </c>
       <c r="AA68" t="n">
-        <v>0.8198</v>
+        <v>0.9599</v>
       </c>
       <c r="AB68" t="n">
-        <v>0.843</v>
+        <v>0.9879</v>
       </c>
       <c r="AC68" t="n">
-        <v>0.8648</v>
+        <v>1.0142</v>
       </c>
       <c r="AD68" t="n">
-        <v>0.8874</v>
+        <v>1.0411</v>
       </c>
       <c r="AE68" t="n">
-        <v>0.9073</v>
+        <v>1.0657</v>
       </c>
       <c r="AF68" t="n">
-        <v>0.9264</v>
+        <v>1.0887</v>
       </c>
       <c r="AG68" t="n">
-        <v>0.9447</v>
+        <v>1.1103</v>
       </c>
       <c r="AH68" t="n">
-        <v>0.9676</v>
+        <v>1.1376</v>
       </c>
       <c r="AI68" t="n">
-        <v>0.9874000000000001</v>
+        <v>1.1605</v>
       </c>
       <c r="AJ68" t="n">
-        <v>1.0073</v>
+        <v>1.1842</v>
       </c>
       <c r="AK68" t="n">
-        <v>1.0254</v>
+        <v>1.2054</v>
       </c>
       <c r="AL68" t="n">
-        <v>1.0352</v>
+        <v>1.2165</v>
       </c>
     </row>
     <row r="69">
@@ -4828,112 +4828,112 @@
         <v>0.1844</v>
       </c>
       <c r="C69" t="n">
-        <v>0.2065</v>
+        <v>0.2139</v>
       </c>
       <c r="D69" t="n">
-        <v>0.2299</v>
+        <v>0.2455</v>
       </c>
       <c r="E69" t="n">
-        <v>0.2532</v>
+        <v>0.2768</v>
       </c>
       <c r="F69" t="n">
-        <v>0.2785</v>
+        <v>0.31</v>
       </c>
       <c r="G69" t="n">
-        <v>0.3015</v>
+        <v>0.3408</v>
       </c>
       <c r="H69" t="n">
-        <v>0.3225</v>
+        <v>0.369</v>
       </c>
       <c r="I69" t="n">
-        <v>0.3436</v>
+        <v>0.3976</v>
       </c>
       <c r="J69" t="n">
-        <v>0.3677</v>
+        <v>0.4286</v>
       </c>
       <c r="K69" t="n">
-        <v>0.3842</v>
+        <v>0.4517</v>
       </c>
       <c r="L69" t="n">
-        <v>0.4093</v>
+        <v>0.4833</v>
       </c>
       <c r="M69" t="n">
-        <v>0.4263</v>
+        <v>0.5063</v>
       </c>
       <c r="N69" t="n">
-        <v>0.4435</v>
+        <v>0.5291</v>
       </c>
       <c r="O69" t="n">
-        <v>0.466</v>
+        <v>0.5574</v>
       </c>
       <c r="P69" t="n">
-        <v>0.4816</v>
+        <v>0.5783</v>
       </c>
       <c r="Q69" t="n">
-        <v>0.4994</v>
+        <v>0.6004</v>
       </c>
       <c r="R69" t="n">
-        <v>0.5169</v>
+        <v>0.6224</v>
       </c>
       <c r="S69" t="n">
-        <v>0.534</v>
+        <v>0.6433</v>
       </c>
       <c r="T69" t="n">
-        <v>0.5456</v>
+        <v>0.6574</v>
       </c>
       <c r="U69" t="n">
-        <v>0.5643</v>
+        <v>0.6798</v>
       </c>
       <c r="V69" t="n">
-        <v>0.5794</v>
+        <v>0.6973</v>
       </c>
       <c r="W69" t="n">
-        <v>0.5951</v>
+        <v>0.7149</v>
       </c>
       <c r="X69" t="n">
-        <v>0.6082</v>
+        <v>0.7294</v>
       </c>
       <c r="Y69" t="n">
-        <v>0.623</v>
+        <v>0.7458</v>
       </c>
       <c r="Z69" t="n">
-        <v>0.6381</v>
+        <v>0.7618</v>
       </c>
       <c r="AA69" t="n">
-        <v>0.6478</v>
+        <v>0.7707000000000001</v>
       </c>
       <c r="AB69" t="n">
-        <v>0.6601</v>
+        <v>0.7832</v>
       </c>
       <c r="AC69" t="n">
-        <v>0.6714</v>
+        <v>0.7937</v>
       </c>
       <c r="AD69" t="n">
-        <v>0.6860000000000001</v>
+        <v>0.8077</v>
       </c>
       <c r="AE69" t="n">
-        <v>0.6914</v>
+        <v>0.8111</v>
       </c>
       <c r="AF69" t="n">
-        <v>0.7049</v>
+        <v>0.8238</v>
       </c>
       <c r="AG69" t="n">
-        <v>0.714</v>
+        <v>0.8300999999999999</v>
       </c>
       <c r="AH69" t="n">
-        <v>0.7246</v>
+        <v>0.8385</v>
       </c>
       <c r="AI69" t="n">
-        <v>0.7348</v>
+        <v>0.8459</v>
       </c>
       <c r="AJ69" t="n">
-        <v>0.7427</v>
+        <v>0.8512</v>
       </c>
       <c r="AK69" t="n">
-        <v>0.7501</v>
+        <v>0.8552</v>
       </c>
       <c r="AL69" t="n">
-        <v>0.7581</v>
+        <v>0.8598</v>
       </c>
     </row>
     <row r="70">
@@ -4946,112 +4946,112 @@
         <v>0.1597</v>
       </c>
       <c r="C70" t="n">
-        <v>0.1744</v>
+        <v>0.1817</v>
       </c>
       <c r="D70" t="n">
-        <v>0.1905</v>
+        <v>0.2055</v>
       </c>
       <c r="E70" t="n">
-        <v>0.2071</v>
+        <v>0.2295</v>
       </c>
       <c r="F70" t="n">
-        <v>0.2214</v>
+        <v>0.2509</v>
       </c>
       <c r="G70" t="n">
-        <v>0.2369</v>
+        <v>0.2725</v>
       </c>
       <c r="H70" t="n">
-        <v>0.25</v>
+        <v>0.2918</v>
       </c>
       <c r="I70" t="n">
-        <v>0.2642</v>
+        <v>0.3112</v>
       </c>
       <c r="J70" t="n">
-        <v>0.2766</v>
+        <v>0.3285</v>
       </c>
       <c r="K70" t="n">
-        <v>0.2888</v>
+        <v>0.3453</v>
       </c>
       <c r="L70" t="n">
-        <v>0.2986</v>
+        <v>0.3589</v>
       </c>
       <c r="M70" t="n">
-        <v>0.3118</v>
+        <v>0.375</v>
       </c>
       <c r="N70" t="n">
-        <v>0.3221</v>
+        <v>0.3879</v>
       </c>
       <c r="O70" t="n">
-        <v>0.3308</v>
+        <v>0.3989</v>
       </c>
       <c r="P70" t="n">
-        <v>0.3164</v>
+        <v>0.3862</v>
       </c>
       <c r="Q70" t="n">
-        <v>0.3501</v>
+        <v>0.421</v>
       </c>
       <c r="R70" t="n">
-        <v>0.3595</v>
+        <v>0.4312</v>
       </c>
       <c r="S70" t="n">
-        <v>0.3702</v>
+        <v>0.4425</v>
       </c>
       <c r="T70" t="n">
-        <v>0.3797</v>
+        <v>0.4517</v>
       </c>
       <c r="U70" t="n">
-        <v>0.3863</v>
+        <v>0.458</v>
       </c>
       <c r="V70" t="n">
-        <v>0.3957</v>
+        <v>0.4668</v>
       </c>
       <c r="W70" t="n">
-        <v>0.4005</v>
+        <v>0.4704</v>
       </c>
       <c r="X70" t="n">
-        <v>0.4058</v>
+        <v>0.4739</v>
       </c>
       <c r="Y70" t="n">
-        <v>0.4135</v>
+        <v>0.4801</v>
       </c>
       <c r="Z70" t="n">
-        <v>0.4181</v>
+        <v>0.483</v>
       </c>
       <c r="AA70" t="n">
-        <v>0.4254</v>
+        <v>0.4888</v>
       </c>
       <c r="AB70" t="n">
-        <v>0.4296</v>
+        <v>0.4905</v>
       </c>
       <c r="AC70" t="n">
-        <v>0.4396</v>
+        <v>0.499</v>
       </c>
       <c r="AD70" t="n">
-        <v>0.4429</v>
+        <v>0.4997</v>
       </c>
       <c r="AE70" t="n">
-        <v>0.4477</v>
+        <v>0.5024999999999999</v>
       </c>
       <c r="AF70" t="n">
-        <v>0.4514</v>
+        <v>0.5041</v>
       </c>
       <c r="AG70" t="n">
-        <v>0.454</v>
+        <v>0.5042</v>
       </c>
       <c r="AH70" t="n">
-        <v>0.4577</v>
+        <v>0.5057</v>
       </c>
       <c r="AI70" t="n">
-        <v>0.464</v>
+        <v>0.5099</v>
       </c>
       <c r="AJ70" t="n">
-        <v>0.4659</v>
+        <v>0.5096000000000001</v>
       </c>
       <c r="AK70" t="n">
-        <v>0.4703</v>
+        <v>0.5119</v>
       </c>
       <c r="AL70" t="n">
-        <v>0.475</v>
+        <v>0.5145999999999999</v>
       </c>
     </row>
     <row r="71">
@@ -5064,112 +5064,112 @@
         <v>0.1715</v>
       </c>
       <c r="C71" t="n">
-        <v>0.1758</v>
+        <v>0.1807</v>
       </c>
       <c r="D71" t="n">
-        <v>0.1867</v>
+        <v>0.1967</v>
       </c>
       <c r="E71" t="n">
-        <v>0.1923</v>
+        <v>0.207</v>
       </c>
       <c r="F71" t="n">
-        <v>0.2013</v>
+        <v>0.2203</v>
       </c>
       <c r="G71" t="n">
-        <v>0.2087</v>
+        <v>0.2314</v>
       </c>
       <c r="H71" t="n">
-        <v>0.2163</v>
+        <v>0.2423</v>
       </c>
       <c r="I71" t="n">
-        <v>0.2218</v>
+        <v>0.2507</v>
       </c>
       <c r="J71" t="n">
-        <v>0.2293</v>
+        <v>0.2609</v>
       </c>
       <c r="K71" t="n">
-        <v>0.2358</v>
+        <v>0.2694</v>
       </c>
       <c r="L71" t="n">
-        <v>0.2415</v>
+        <v>0.277</v>
       </c>
       <c r="M71" t="n">
-        <v>0.2468</v>
+        <v>0.2835</v>
       </c>
       <c r="N71" t="n">
-        <v>0.2526</v>
+        <v>0.2907</v>
       </c>
       <c r="O71" t="n">
-        <v>0.2603</v>
+        <v>0.2992</v>
       </c>
       <c r="P71" t="n">
-        <v>0.2626</v>
+        <v>0.3018</v>
       </c>
       <c r="Q71" t="n">
-        <v>0.2656</v>
+        <v>0.305</v>
       </c>
       <c r="R71" t="n">
-        <v>0.271</v>
+        <v>0.3106</v>
       </c>
       <c r="S71" t="n">
-        <v>0.275</v>
+        <v>0.3147</v>
       </c>
       <c r="T71" t="n">
-        <v>0.2814</v>
+        <v>0.3206</v>
       </c>
       <c r="U71" t="n">
-        <v>0.2837</v>
+        <v>0.3223</v>
       </c>
       <c r="V71" t="n">
-        <v>0.2896</v>
+        <v>0.3279</v>
       </c>
       <c r="W71" t="n">
-        <v>0.2908</v>
+        <v>0.3282</v>
       </c>
       <c r="X71" t="n">
-        <v>0.2937</v>
+        <v>0.3303</v>
       </c>
       <c r="Y71" t="n">
-        <v>0.2983</v>
+        <v>0.334</v>
       </c>
       <c r="Z71" t="n">
-        <v>0.3009</v>
+        <v>0.3354</v>
       </c>
       <c r="AA71" t="n">
-        <v>0.3039</v>
+        <v>0.3377</v>
       </c>
       <c r="AB71" t="n">
-        <v>0.3064</v>
+        <v>0.339</v>
       </c>
       <c r="AC71" t="n">
-        <v>0.3077</v>
+        <v>0.3389</v>
       </c>
       <c r="AD71" t="n">
-        <v>0.3123</v>
+        <v>0.3428</v>
       </c>
       <c r="AE71" t="n">
-        <v>0.3138</v>
+        <v>0.3433</v>
       </c>
       <c r="AF71" t="n">
-        <v>0.3157</v>
+        <v>0.3438</v>
       </c>
       <c r="AG71" t="n">
-        <v>0.3202</v>
+        <v>0.3472</v>
       </c>
       <c r="AH71" t="n">
-        <v>0.3194</v>
+        <v>0.3454</v>
       </c>
       <c r="AI71" t="n">
-        <v>0.3224</v>
+        <v>0.3472</v>
       </c>
       <c r="AJ71" t="n">
-        <v>0.3233</v>
+        <v>0.3471</v>
       </c>
       <c r="AK71" t="n">
-        <v>0.3249</v>
+        <v>0.3477</v>
       </c>
       <c r="AL71" t="n">
-        <v>0.3269</v>
+        <v>0.3486</v>
       </c>
     </row>
     <row r="72">

</xml_diff>